<commit_message>
Grace sales tracker r2: Ralph's answers, House of Rameau inventory
- VERSIONS.md v2 in Grace's looser wording (Ralph: 'Use looser wording');
  check.py now requires a named library hook base, not word for word
- Promoted column: TikTok's ad label = brand-paid promotion (Ralph)
- houseoframeau/: shared account via Composio TikTok, 26 public videos,
  8 shop videos, refresh steps
- HOOKS.md exception for winners' new versions; skill updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SJD4VaSy9o4r7BFp61EpGh
</commit_message>
<xml_diff>
--- a/grace/winners/winners.xlsx
+++ b/grace/winners/winners.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W7"/>
+  <dimension ref="A1:X7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -437,21 +437,22 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="35" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
     <col width="35" customWidth="1" min="14" max="14"/>
-    <col width="55" customWidth="1" min="15" max="15"/>
-    <col width="70" customWidth="1" min="16" max="16"/>
-    <col width="30" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="35" customWidth="1" min="15" max="15"/>
+    <col width="55" customWidth="1" min="16" max="16"/>
+    <col width="70" customWidth="1" min="17" max="17"/>
+    <col width="30" customWidth="1" min="18" max="18"/>
     <col width="14" customWidth="1" min="19" max="19"/>
     <col width="14" customWidth="1" min="20" max="20"/>
     <col width="14" customWidth="1" min="21" max="21"/>
     <col width="14" customWidth="1" min="22" max="22"/>
     <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -487,85 +488,90 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Promoted</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Faceless</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Format</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Hook (first line said)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Hook type</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Library hook</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>On-screen text</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Pain point</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Problem the product solves</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Why it converted (our read)</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Script used (as posted)</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Link to video</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Product link</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Saves</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Shares</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Length (s)</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Our job folder</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
@@ -598,79 +604,84 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>Yes, by the brand (TikTok ad label)</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Hands + voiceover, AI, reply-to-comment video (marble bathroom, oil pour vs roll-on)</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>The only thing I hate about Castor oil is how thick and messy it is.</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Objection / Problem Callout</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>own line</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Reply-to-comment sticker: "I think we all need castor oil" (@umi3728)</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Castor oil is thick, messy and drips on your fingers, and the smell lingers.</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>A roll-on bottle with a rose quartz roller: no pouring, no oily fingers, put it exactly where you want (brows, cuticles, skin, hair).</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>Fastest start of the 6 (763 views a day). It replies to a real comment from her viral cradle-cap video, so it reaches people who already asked for castor oil (warm audience). Before/after messy pour vs clean roll is the proof. Grace's own wording ("freaking genius", "I'mma do y'all a favor") sounds like her, not an ad.</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>The only thing I hate about Castor oil is how thick and messy it is. And let's be for real, the smell isn't exactly something you want lingering all day. But if you know, you know, Castor oil is liquid gold. And this roll on. Freaking ingenious. No pouring, no oily fingers. Just roll it exactly where you want it. It's USDA organic, cold pressed and hexane free with a rose quartz roller. I'mma do y'all a favor and link it in the orange car. If you want condition brows, softer cuticles, moisturize skin and hair, growing longer, smoother, and shinier, you know what to do.</t>
         </is>
       </c>
-      <c r="Q2" s="2" t="inlineStr">
+      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>https://www.tiktok.com/@shewiththeglow/video/7697844264050511135</t>
         </is>
       </c>
-      <c r="R2" s="2" t="inlineStr">
+      <c r="S2" s="2" t="inlineStr">
         <is>
           <t>https://shop.tiktok.com/us/pdp/castor-castor-oil-roll-on-usda-organic-50ml-easy-application/1732039499743138513</t>
         </is>
       </c>
-      <c r="S2" s="2" t="n">
+      <c r="T2" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="T2" s="2" t="n">
+      <c r="U2" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="U2" s="2" t="n">
+      <c r="V2" s="2" t="n">
         <v>31</v>
       </c>
-      <c r="V2" s="2" t="inlineStr">
+      <c r="W2" s="2" t="inlineStr">
         <is>
           <t>ugc/bodyj-castor-rollon/v2g (Grace's own script, word for word)</t>
         </is>
       </c>
-      <c r="W2" s="2" t="inlineStr"/>
+      <c r="X2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -699,79 +710,84 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
+          <t>Yes, by the brand (TikTok ad label)</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Hands + hand-free moving shots + voiceover, AI (pantry, garage, dog in hallway)</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Listen, when it gets cold outside, mice start looking for somewhere warm, and your house might be exactly what they're looking for.</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Time Pressure (Grace's rewording of H130)</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>own line</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>the last thing you want in your pantry... 😳</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>Mice moving in when it gets cold, and only finding out from droppings in the pantry; not wanting poison or traps around kids and pets.</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="O3" s="2" t="inlineStr">
         <is>
           <t>Peppermint + cinnamon oil pouches you drop where mice get in; no toxic chemicals, no traps to empty, 12 per bag, up to 3 months each.</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
+      <c r="P3" s="2" t="inlineStr">
         <is>
           <t>Prevention before a deadline (cold weather) with a gross, visual payoff (droppings on the shelf). Removes the two big objections in one line each: safe around kids and pets, no traps to empty. The count + "grab two bags and do the whole house" pushes more than one unit.</t>
         </is>
       </c>
-      <c r="P3" s="2" t="inlineStr">
+      <c r="Q3" s="2" t="inlineStr">
         <is>
           <t>Listen, when it gets cold outside, mice start looking for somewhere warm, and your house might be exactly what they're looking for. And you won't even know until there are droppings in your pantry. So these let them out now. Just drop one wherever they get in. The pantry, under the sink, the garage, even the car. It's peppermint and cinnamon oil, so it smells fresh to us, but for mice, they don't like it. No toxic chemicals, so it's safe around kids and pets. And honestly, the best part, there's no traps to empty. There are 12 in the bag, and each one lasts up to three months. So grab two bags and do the whole house before the cold hits. I linked them below in the orange cart for you.</t>
         </is>
       </c>
-      <c r="Q3" s="2" t="inlineStr">
+      <c r="R3" s="2" t="inlineStr">
         <is>
           <t>https://www.tiktok.com/@shewiththeglow/video/7696617399759555871</t>
         </is>
       </c>
-      <c r="R3" s="2" t="inlineStr">
+      <c r="S3" s="2" t="inlineStr">
         <is>
           <t>https://shop.tiktok.com/us/pdp/sofyre-mouse-repellent-pouches-natural-rodent-deterrent/1729505002971305054</t>
         </is>
-      </c>
-      <c r="S3" s="2" t="n">
-        <v>5</v>
       </c>
       <c r="T3" s="2" t="n">
         <v>5</v>
       </c>
       <c r="U3" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="V3" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="V3" s="2" t="inlineStr">
+      <c r="W3" s="2" t="inlineStr">
         <is>
           <t>ugc/sofyre-rodent-pouches (r1 VO; Grace opened with "Listen," and reworded the hook when posting)</t>
         </is>
       </c>
-      <c r="W3" s="2" t="inlineStr"/>
+      <c r="X3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -800,79 +816,84 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Hands + voiceover, AI (overhead family table, cards being played)</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>You know game night is a wack when everyone's sitting around staring at their phones.</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>Recognition (Grace's rewording of H062)</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>own line</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>POV: you finally found a game everyone wants to play....</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>Game night dies: everyone on their phones, or the game drags so long people lose interest.</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr">
         <is>
           <t>A 60-second rock-paper-scissors card game, no waiting your turn, 2 to 8 players, easy to learn on the spot.</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr">
+      <c r="P4" s="2" t="inlineStr">
         <is>
           <t>Opens on a scene every family knows (phones at the table), then the rules are shown, not explained, so the viewer understands the game in 10 seconds. Thanksgiving gives the deadline, and "one for your house and one for your grandma's" sells two. Gift-able, low price.</t>
         </is>
       </c>
-      <c r="P4" s="2" t="inlineStr">
+      <c r="Q4" s="2" t="inlineStr">
         <is>
           <t>You know game night is a wack when everyone's sitting around staring at their phones. Or when the game drags so long that everybody loses interest. This game fixes that real quick. It's called Throw Hands and think Rock, Paper, Scissors, but with cards and absolutely no waiting your turn. You slap down the card that beats the last one. Rock beat Scissors, paper beats rock, and Scissors beats paper. First person to get rid of all their cards wins. And with rounds lasting just 60 seconds, good luck just playing one round. Holiday fun is coming up, so grab one for your house and one for your grandma's. I linked it in the orange cart for you.</t>
         </is>
       </c>
-      <c r="Q4" s="2" t="inlineStr">
+      <c r="R4" s="2" t="inlineStr">
         <is>
           <t>https://www.tiktok.com/@shewiththeglow/video/7696627904985304351</t>
         </is>
       </c>
-      <c r="R4" s="2" t="inlineStr">
+      <c r="S4" s="2" t="inlineStr">
         <is>
           <t>https://shop.tiktok.com/us/pdp/fast-fun-card-game-for-2-8-players-perfect-for-parties/1732271777612075081</t>
         </is>
-      </c>
-      <c r="S4" s="2" t="n">
-        <v>1</v>
       </c>
       <c r="T4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="U4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V4" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="V4" s="2" t="inlineStr">
+      <c r="W4" s="2" t="inlineStr">
         <is>
           <t>ugc/throw-hands-rps (r2b; Grace reworded the VO when posting)</t>
         </is>
       </c>
-      <c r="W4" s="2" t="inlineStr"/>
+      <c r="X4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -901,79 +922,84 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
+          <t>Yes, by the brand (TikTok ad label)</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Hands + voiceover, AI (bedroom at night, box + dilator close-ups)</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>This is for the people who always end up on the couch because somebody will not stop snoring.</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>Identity</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>H061</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>POV: someone's snoring is ruining your sleep 😭</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>Losing sleep (or ending up on the couch) because the person next to you snores; nudging, earplugs and mouth tape did not fix it.</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="O5" s="2" t="inlineStr">
         <is>
           <t>A tiny clear nasal dilator opens the nose so they snore less; the starter pack has all 3 sizes so you find the fit.</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr">
+      <c r="P5" s="2" t="inlineStr">
         <is>
           <t>Speaks to the person who suffers (the partner), not the snorer, so the buyer is the viewer. Lists what they already tried, then shows a small, cheap-feeling fix. Holiday shared rooms gives a reason to buy now. Most views of the 6 (3.9k) but the most views per sale: the broad pain gets reach, fewer of those viewers are ready to buy.</t>
         </is>
       </c>
-      <c r="P5" s="2" t="inlineStr">
+      <c r="Q5" s="2" t="inlineStr">
         <is>
           <t>This is for the people who always end up on the couch because somebody will not stop snoring. You've tried nudging them, earplugs, and even mouth tape. This is mute, a tiny clear dilator that gently opens your nose. The starter pack has all three sizes and each one lasts up to 10 nights. Imagine actually getting some sleep instead of listening to snoring all night. And with the holiday travel coming up, this is worth packing for shared rooms. And you can find the mute starter pack a link below in the orange cart.</t>
         </is>
       </c>
-      <c r="Q5" s="2" t="inlineStr">
+      <c r="R5" s="2" t="inlineStr">
         <is>
           <t>https://www.tiktok.com/@shewiththeglow/video/7696231728855223582</t>
         </is>
       </c>
-      <c r="R5" s="2" t="inlineStr">
+      <c r="S5" s="2" t="inlineStr">
         <is>
           <t>https://shop.tiktok.com/us/pdp/mute-nasal-dilator-starter-pack-reduces-snoring-3-sizes/1732240917356122930</t>
         </is>
       </c>
-      <c r="S5" s="2" t="n">
+      <c r="T5" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="T5" s="2" t="n">
+      <c r="U5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="U5" s="2" t="n">
+      <c r="V5" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="V5" s="2" t="inlineStr">
+      <c r="W5" s="2" t="inlineStr">
         <is>
           <t>ugc/mute-nasal-dilator (r4 VO; Grace dropped the 75% trial stat and the 2 a.m. joke when posting)</t>
         </is>
       </c>
-      <c r="W5" s="2" t="inlineStr"/>
+      <c r="X5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1002,79 +1028,84 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
+          <t>Yes, by the brand (TikTok ad label)</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Hands + voiceover, AI (POV through the windshield at night, glasses on the dash)</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>I wish someone thought of this sooner, because blinding headlights at night time, that's a whole different scary.</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>Problem/Solution (close to H010)</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>own line</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>blinding headlights at night are SCARY 😩</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>Being blinded by bright headlights at night, squinting at the lane lines; worse if you already wear glasses.</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="O6" s="2" t="inlineStr">
         <is>
           <t>Yellow-lens night driving glasses that fit over regular glasses, with side windows so glare cannot sneak in from the side.</t>
         </is>
       </c>
-      <c r="O6" s="2" t="inlineStr">
+      <c r="P6" s="2" t="inlineStr">
         <is>
           <t>Fewest views per sale of Grace's 5 (463 views, 1 sale). The fear is specific and visual (the white glare on screen), the viewer pictures their own drive home, and the clocks-go-back date (Nov 1) is real urgency. "Fit right over your regular ones" answers the glasses-wearer objection before they think it. Multi-unit ask: "grab one for a friend".</t>
         </is>
       </c>
-      <c r="P6" s="2" t="inlineStr">
+      <c r="Q6" s="2" t="inlineStr">
         <is>
           <t>I wish someone thought of this sooner, because blinding headlights at night time, that's a whole different scary. You're squinting at the lane lines, just hoping you're still in your lane. And wearing glasses that makes it even worse. These are night driving glasses that fit right over your regular ones. The yellow lenses are designed to help reduce glare from oncoming headlights. And there's a little window on each side so the glare can't even sneak in from the side. Now the clocks do go back on November 1st, which means darker drives home. Getting a pair of these is so worth it. And if you're feeling generous, grab one for a friend too. It's linked below in the orange cart.</t>
         </is>
       </c>
-      <c r="Q6" s="2" t="inlineStr">
+      <c r="R6" s="2" t="inlineStr">
         <is>
           <t>https://www.tiktok.com/@shewiththeglow/video/7696285070046301470</t>
         </is>
       </c>
-      <c r="R6" s="2" t="inlineStr">
+      <c r="S6" s="2" t="inlineStr">
         <is>
           <t>https://shop.tiktok.com/us/pdp/night-vision-driving-glasses-anti-glare-polarized-lenses/1731941490512139199</t>
         </is>
       </c>
-      <c r="S6" s="2" t="n">
+      <c r="T6" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="T6" s="2" t="n">
+      <c r="U6" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="U6" s="2" t="n">
+      <c r="V6" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="V6" s="2" t="inlineStr">
+      <c r="W6" s="2" t="inlineStr">
         <is>
           <t>ugc/night-driving-glasses/v2 (Grace's V1 script; she added "I wish someone thought of this sooner" at the start)</t>
         </is>
       </c>
-      <c r="W6" s="2" t="inlineStr"/>
+      <c r="X6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1103,79 +1134,84 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
           <t>No (AI man talking to camera)</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Talking head, AI, lip-synced, home office, product worn and held to camera</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>If this is your year to level up, do not scroll past this.</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Identity (callout)</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>own line</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>the necklace for your abundance era...✨</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>Wanting to "level up" (money, confidence) this year and wanting something that reminds you every day.</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="O7" s="2" t="inlineStr">
         <is>
           <t>A genuine tiger eye pendant on black and gold beads, an everyday reminder of abundance and confidence (identity product, not a fix).</t>
         </is>
       </c>
-      <c r="O7" s="2" t="inlineStr">
+      <c r="P7" s="2" t="inlineStr">
         <is>
           <t>1 sale on 61 views: tiny sample, so this is a lead, not proof. Short (13s) and fast. Identity hook ("if this is your year to level up") lets the buyer see themselves in it; close-ups show the stone catching the light (proof of quality), "heavy, solid, the real deal". Watch: "these keep selling out" is a scarcity claim we cannot back; keep it out of new versions unless the shop shows it.</t>
         </is>
       </c>
-      <c r="P7" s="2" t="inlineStr">
+      <c r="Q7" s="2" t="inlineStr">
         <is>
           <t>If this is your year to level up, do not scroll past this. This isn't just jewelry, it's your everyday reminder to attract wealth and abundance. Genuine tiger eye, look out, catches the light. Heavy, solid, the real deal. Black and gold beads all the way around. These keep selling out. Links down there, grab yours. Thank me later.</t>
         </is>
       </c>
-      <c r="Q7" s="2" t="inlineStr">
+      <c r="R7" s="2" t="inlineStr">
         <is>
           <t>https://www.tiktok.com/@houseoframeau/video/7685441537894780190</t>
         </is>
       </c>
-      <c r="R7" s="2" t="inlineStr">
+      <c r="S7" s="2" t="inlineStr">
         <is>
           <t>https://shop.tiktok.com/us/pdp/arpurraina-money-attraction-necklace-tiger-eye-pendant/1732052135957598240</t>
         </is>
       </c>
-      <c r="S7" s="2" t="n">
+      <c r="T7" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="T7" s="2" t="n">
+      <c r="U7" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="U7" s="2" t="n">
+      <c r="V7" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="V7" s="2" t="inlineStr">
+      <c r="W7" s="2" t="inlineStr">
         <is>
           <t>houseoframeau account (not a Mymobileworld job folder)</t>
         </is>
       </c>
-      <c r="W7" s="2" t="inlineStr"/>
+      <c r="X7" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sales tracker: BodyJ castor roll-on now 2 sales (Grace)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SJD4VaSy9o4r7BFp61EpGh
</commit_message>
<xml_diff>
--- a/grace/winners/winners.xlsx
+++ b/grace/winners/winners.xlsx
@@ -594,13 +594,13 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1144</v>
+        <v>1538</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>1144</v>
+        <v>769</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -1127,10 +1127,10 @@
         <v>1</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Sales tracker: BodyJ castor roll-on now 3 sales (Grace)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SJD4VaSy9o4r7BFp61EpGh
</commit_message>
<xml_diff>
--- a/grace/winners/winners.xlsx
+++ b/grace/winners/winners.xlsx
@@ -594,13 +594,13 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1538</v>
+        <v>1578</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>769</v>
+        <v>526</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Sales tracker: Voice column; castor seller is Grace's own voice (Ralph)
PATTERNS #10, PLAYBOOK lesson, VERSIONS: Grace records the VO herself.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SJD4VaSy9o4r7BFp61EpGh
</commit_message>
<xml_diff>
--- a/grace/winners/winners.xlsx
+++ b/grace/winners/winners.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X7"/>
+  <dimension ref="A1:Y7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -438,21 +438,22 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="35" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
     <col width="35" customWidth="1" min="15" max="15"/>
-    <col width="55" customWidth="1" min="16" max="16"/>
-    <col width="70" customWidth="1" min="17" max="17"/>
-    <col width="30" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="35" customWidth="1" min="16" max="16"/>
+    <col width="55" customWidth="1" min="17" max="17"/>
+    <col width="70" customWidth="1" min="18" max="18"/>
+    <col width="30" customWidth="1" min="19" max="19"/>
     <col width="14" customWidth="1" min="20" max="20"/>
     <col width="14" customWidth="1" min="21" max="21"/>
     <col width="14" customWidth="1" min="22" max="22"/>
     <col width="14" customWidth="1" min="23" max="23"/>
     <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,80 +499,85 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>Voice</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Format</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Hook (first line said)</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Hook type</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Library hook</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>On-screen text</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Pain point</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Problem the product solves</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Why it converted (our read)</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Script used (as posted)</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Link to video</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Product link</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Saves</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Shares</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Length (s)</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Our job folder</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
@@ -614,74 +620,79 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
+          <t>Grace's own voice (Ralph 2026-10-20)</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
           <t>Hands + voiceover, AI, reply-to-comment video (marble bathroom, oil pour vs roll-on)</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>The only thing I hate about Castor oil is how thick and messy it is.</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Objection / Problem Callout</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>own line</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Reply-to-comment sticker: "I think we all need castor oil" (@umi3728)</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>Castor oil is thick, messy and drips on your fingers, and the smell lingers.</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>A roll-on bottle with a rose quartz roller: no pouring, no oily fingers, put it exactly where you want (brows, cuticles, skin, hair).</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>Fastest start of the 6 (763 views a day). It replies to a real comment from her viral cradle-cap video, so it reaches people who already asked for castor oil (warm audience). Before/after messy pour vs clean roll is the proof. Grace's own wording ("freaking genius", "I'mma do y'all a favor") sounds like her, not an ad.</t>
         </is>
       </c>
-      <c r="Q2" s="2" t="inlineStr">
+      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>The only thing I hate about Castor oil is how thick and messy it is. And let's be for real, the smell isn't exactly something you want lingering all day. But if you know, you know, Castor oil is liquid gold. And this roll on. Freaking ingenious. No pouring, no oily fingers. Just roll it exactly where you want it. It's USDA organic, cold pressed and hexane free with a rose quartz roller. I'mma do y'all a favor and link it in the orange car. If you want condition brows, softer cuticles, moisturize skin and hair, growing longer, smoother, and shinier, you know what to do.</t>
         </is>
       </c>
-      <c r="R2" s="2" t="inlineStr">
+      <c r="S2" s="2" t="inlineStr">
         <is>
           <t>https://www.tiktok.com/@shewiththeglow/video/7697844264050511135</t>
         </is>
       </c>
-      <c r="S2" s="2" t="inlineStr">
+      <c r="T2" s="2" t="inlineStr">
         <is>
           <t>https://shop.tiktok.com/us/pdp/castor-castor-oil-roll-on-usda-organic-50ml-easy-application/1732039499743138513</t>
         </is>
       </c>
-      <c r="T2" s="2" t="n">
+      <c r="U2" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="U2" s="2" t="n">
+      <c r="V2" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="V2" s="2" t="n">
+      <c r="W2" s="2" t="n">
         <v>31</v>
       </c>
-      <c r="W2" s="2" t="inlineStr">
+      <c r="X2" s="2" t="inlineStr">
         <is>
           <t>ugc/bodyj-castor-rollon/v2g (Grace's own script, word for word)</t>
         </is>
       </c>
-      <c r="X2" s="2" t="inlineStr"/>
+      <c r="Y2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -720,74 +731,79 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
+          <t>likely Grace's own voice: posted words differ from our ElevenLabs file (to confirm)</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
           <t>Hands + hand-free moving shots + voiceover, AI (pantry, garage, dog in hallway)</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Listen, when it gets cold outside, mice start looking for somewhere warm, and your house might be exactly what they're looking for.</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>Time Pressure (Grace's rewording of H130)</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>own line</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>the last thing you want in your pantry... 😳</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="O3" s="2" t="inlineStr">
         <is>
           <t>Mice moving in when it gets cold, and only finding out from droppings in the pantry; not wanting poison or traps around kids and pets.</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
+      <c r="P3" s="2" t="inlineStr">
         <is>
           <t>Peppermint + cinnamon oil pouches you drop where mice get in; no toxic chemicals, no traps to empty, 12 per bag, up to 3 months each.</t>
         </is>
       </c>
-      <c r="P3" s="2" t="inlineStr">
+      <c r="Q3" s="2" t="inlineStr">
         <is>
           <t>Prevention before a deadline (cold weather) with a gross, visual payoff (droppings on the shelf). Removes the two big objections in one line each: safe around kids and pets, no traps to empty. The count + "grab two bags and do the whole house" pushes more than one unit.</t>
         </is>
       </c>
-      <c r="Q3" s="2" t="inlineStr">
+      <c r="R3" s="2" t="inlineStr">
         <is>
           <t>Listen, when it gets cold outside, mice start looking for somewhere warm, and your house might be exactly what they're looking for. And you won't even know until there are droppings in your pantry. So these let them out now. Just drop one wherever they get in. The pantry, under the sink, the garage, even the car. It's peppermint and cinnamon oil, so it smells fresh to us, but for mice, they don't like it. No toxic chemicals, so it's safe around kids and pets. And honestly, the best part, there's no traps to empty. There are 12 in the bag, and each one lasts up to three months. So grab two bags and do the whole house before the cold hits. I linked them below in the orange cart for you.</t>
         </is>
       </c>
-      <c r="R3" s="2" t="inlineStr">
+      <c r="S3" s="2" t="inlineStr">
         <is>
           <t>https://www.tiktok.com/@shewiththeglow/video/7696617399759555871</t>
         </is>
       </c>
-      <c r="S3" s="2" t="inlineStr">
+      <c r="T3" s="2" t="inlineStr">
         <is>
           <t>https://shop.tiktok.com/us/pdp/sofyre-mouse-repellent-pouches-natural-rodent-deterrent/1729505002971305054</t>
         </is>
-      </c>
-      <c r="T3" s="2" t="n">
-        <v>5</v>
       </c>
       <c r="U3" s="2" t="n">
         <v>5</v>
       </c>
       <c r="V3" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="W3" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="W3" s="2" t="inlineStr">
+      <c r="X3" s="2" t="inlineStr">
         <is>
           <t>ugc/sofyre-rodent-pouches (r1 VO; Grace opened with "Listen," and reworded the hook when posting)</t>
         </is>
       </c>
-      <c r="X3" s="2" t="inlineStr"/>
+      <c r="Y3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -826,74 +842,79 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
+          <t>likely Grace's own voice: posted words differ from our ElevenLabs file (to confirm)</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
           <t>Hands + voiceover, AI (overhead family table, cards being played)</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>You know game night is a wack when everyone's sitting around staring at their phones.</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>Recognition (Grace's rewording of H062)</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>own line</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>POV: you finally found a game everyone wants to play....</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr">
         <is>
           <t>Game night dies: everyone on their phones, or the game drags so long people lose interest.</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr">
+      <c r="P4" s="2" t="inlineStr">
         <is>
           <t>A 60-second rock-paper-scissors card game, no waiting your turn, 2 to 8 players, easy to learn on the spot.</t>
         </is>
       </c>
-      <c r="P4" s="2" t="inlineStr">
+      <c r="Q4" s="2" t="inlineStr">
         <is>
           <t>Opens on a scene every family knows (phones at the table), then the rules are shown, not explained, so the viewer understands the game in 10 seconds. Thanksgiving gives the deadline, and "one for your house and one for your grandma's" sells two. Gift-able, low price.</t>
         </is>
       </c>
-      <c r="Q4" s="2" t="inlineStr">
+      <c r="R4" s="2" t="inlineStr">
         <is>
           <t>You know game night is a wack when everyone's sitting around staring at their phones. Or when the game drags so long that everybody loses interest. This game fixes that real quick. It's called Throw Hands and think Rock, Paper, Scissors, but with cards and absolutely no waiting your turn. You slap down the card that beats the last one. Rock beat Scissors, paper beats rock, and Scissors beats paper. First person to get rid of all their cards wins. And with rounds lasting just 60 seconds, good luck just playing one round. Holiday fun is coming up, so grab one for your house and one for your grandma's. I linked it in the orange cart for you.</t>
         </is>
       </c>
-      <c r="R4" s="2" t="inlineStr">
+      <c r="S4" s="2" t="inlineStr">
         <is>
           <t>https://www.tiktok.com/@shewiththeglow/video/7696627904985304351</t>
         </is>
       </c>
-      <c r="S4" s="2" t="inlineStr">
+      <c r="T4" s="2" t="inlineStr">
         <is>
           <t>https://shop.tiktok.com/us/pdp/fast-fun-card-game-for-2-8-players-perfect-for-parties/1732271777612075081</t>
         </is>
-      </c>
-      <c r="T4" s="2" t="n">
-        <v>1</v>
       </c>
       <c r="U4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="V4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W4" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="W4" s="2" t="inlineStr">
+      <c r="X4" s="2" t="inlineStr">
         <is>
           <t>ugc/throw-hands-rps (r2b; Grace reworded the VO when posting)</t>
         </is>
       </c>
-      <c r="X4" s="2" t="inlineStr"/>
+      <c r="Y4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -932,74 +953,79 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
+          <t>likely Grace's own voice: posted words differ from our ElevenLabs file (to confirm)</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
           <t>Hands + voiceover, AI (bedroom at night, box + dilator close-ups)</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>This is for the people who always end up on the couch because somebody will not stop snoring.</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>Identity</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>H061</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>POV: someone's snoring is ruining your sleep 😭</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="O5" s="2" t="inlineStr">
         <is>
           <t>Losing sleep (or ending up on the couch) because the person next to you snores; nudging, earplugs and mouth tape did not fix it.</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr">
+      <c r="P5" s="2" t="inlineStr">
         <is>
           <t>A tiny clear nasal dilator opens the nose so they snore less; the starter pack has all 3 sizes so you find the fit.</t>
         </is>
       </c>
-      <c r="P5" s="2" t="inlineStr">
+      <c r="Q5" s="2" t="inlineStr">
         <is>
           <t>Speaks to the person who suffers (the partner), not the snorer, so the buyer is the viewer. Lists what they already tried, then shows a small, cheap-feeling fix. Holiday shared rooms gives a reason to buy now. Most views of the 6 (3.9k) but the most views per sale: the broad pain gets reach, fewer of those viewers are ready to buy.</t>
         </is>
       </c>
-      <c r="Q5" s="2" t="inlineStr">
+      <c r="R5" s="2" t="inlineStr">
         <is>
           <t>This is for the people who always end up on the couch because somebody will not stop snoring. You've tried nudging them, earplugs, and even mouth tape. This is mute, a tiny clear dilator that gently opens your nose. The starter pack has all three sizes and each one lasts up to 10 nights. Imagine actually getting some sleep instead of listening to snoring all night. And with the holiday travel coming up, this is worth packing for shared rooms. And you can find the mute starter pack a link below in the orange cart.</t>
         </is>
       </c>
-      <c r="R5" s="2" t="inlineStr">
+      <c r="S5" s="2" t="inlineStr">
         <is>
           <t>https://www.tiktok.com/@shewiththeglow/video/7696231728855223582</t>
         </is>
       </c>
-      <c r="S5" s="2" t="inlineStr">
+      <c r="T5" s="2" t="inlineStr">
         <is>
           <t>https://shop.tiktok.com/us/pdp/mute-nasal-dilator-starter-pack-reduces-snoring-3-sizes/1732240917356122930</t>
         </is>
       </c>
-      <c r="T5" s="2" t="n">
+      <c r="U5" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="U5" s="2" t="n">
+      <c r="V5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="V5" s="2" t="n">
+      <c r="W5" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="W5" s="2" t="inlineStr">
+      <c r="X5" s="2" t="inlineStr">
         <is>
           <t>ugc/mute-nasal-dilator (r4 VO; Grace dropped the 75% trial stat and the 2 a.m. joke when posting)</t>
         </is>
       </c>
-      <c r="X5" s="2" t="inlineStr"/>
+      <c r="Y5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1038,74 +1064,79 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
+          <t>likely Grace's own voice: posted words differ from our ElevenLabs file (to confirm)</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
           <t>Hands + voiceover, AI (POV through the windshield at night, glasses on the dash)</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>I wish someone thought of this sooner, because blinding headlights at night time, that's a whole different scary.</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>Problem/Solution (close to H010)</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>own line</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>blinding headlights at night are SCARY 😩</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="O6" s="2" t="inlineStr">
         <is>
           <t>Being blinded by bright headlights at night, squinting at the lane lines; worse if you already wear glasses.</t>
         </is>
       </c>
-      <c r="O6" s="2" t="inlineStr">
+      <c r="P6" s="2" t="inlineStr">
         <is>
           <t>Yellow-lens night driving glasses that fit over regular glasses, with side windows so glare cannot sneak in from the side.</t>
         </is>
       </c>
-      <c r="P6" s="2" t="inlineStr">
+      <c r="Q6" s="2" t="inlineStr">
         <is>
           <t>Fewest views per sale of Grace's 5 (463 views, 1 sale). The fear is specific and visual (the white glare on screen), the viewer pictures their own drive home, and the clocks-go-back date (Nov 1) is real urgency. "Fit right over your regular ones" answers the glasses-wearer objection before they think it. Multi-unit ask: "grab one for a friend".</t>
         </is>
       </c>
-      <c r="Q6" s="2" t="inlineStr">
+      <c r="R6" s="2" t="inlineStr">
         <is>
           <t>I wish someone thought of this sooner, because blinding headlights at night time, that's a whole different scary. You're squinting at the lane lines, just hoping you're still in your lane. And wearing glasses that makes it even worse. These are night driving glasses that fit right over your regular ones. The yellow lenses are designed to help reduce glare from oncoming headlights. And there's a little window on each side so the glare can't even sneak in from the side. Now the clocks do go back on November 1st, which means darker drives home. Getting a pair of these is so worth it. And if you're feeling generous, grab one for a friend too. It's linked below in the orange cart.</t>
         </is>
       </c>
-      <c r="R6" s="2" t="inlineStr">
+      <c r="S6" s="2" t="inlineStr">
         <is>
           <t>https://www.tiktok.com/@shewiththeglow/video/7696285070046301470</t>
         </is>
       </c>
-      <c r="S6" s="2" t="inlineStr">
+      <c r="T6" s="2" t="inlineStr">
         <is>
           <t>https://shop.tiktok.com/us/pdp/night-vision-driving-glasses-anti-glare-polarized-lenses/1731941490512139199</t>
         </is>
       </c>
-      <c r="T6" s="2" t="n">
+      <c r="U6" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="U6" s="2" t="n">
+      <c r="V6" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="V6" s="2" t="n">
+      <c r="W6" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="W6" s="2" t="inlineStr">
+      <c r="X6" s="2" t="inlineStr">
         <is>
           <t>ugc/night-driving-glasses/v2 (Grace's V1 script; she added "I wish someone thought of this sooner" at the start)</t>
         </is>
       </c>
-      <c r="X6" s="2" t="inlineStr"/>
+      <c r="Y6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1144,74 +1175,79 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
+          <t>not known yet</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
           <t>Talking head, AI, lip-synced, home office, product worn and held to camera</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>If this is your year to level up, do not scroll past this.</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Identity (callout)</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>own line</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>the necklace for your abundance era...✨</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="O7" s="2" t="inlineStr">
         <is>
           <t>Wanting to "level up" (money, confidence) this year and wanting something that reminds you every day.</t>
         </is>
       </c>
-      <c r="O7" s="2" t="inlineStr">
+      <c r="P7" s="2" t="inlineStr">
         <is>
           <t>A genuine tiger eye pendant on black and gold beads, an everyday reminder of abundance and confidence (identity product, not a fix).</t>
         </is>
       </c>
-      <c r="P7" s="2" t="inlineStr">
+      <c r="Q7" s="2" t="inlineStr">
         <is>
           <t>1 sale on 61 views: tiny sample, so this is a lead, not proof. Short (13s) and fast. Identity hook ("if this is your year to level up") lets the buyer see themselves in it; close-ups show the stone catching the light (proof of quality), "heavy, solid, the real deal". Watch: "these keep selling out" is a scarcity claim we cannot back; keep it out of new versions unless the shop shows it.</t>
         </is>
       </c>
-      <c r="Q7" s="2" t="inlineStr">
+      <c r="R7" s="2" t="inlineStr">
         <is>
           <t>If this is your year to level up, do not scroll past this. This isn't just jewelry, it's your everyday reminder to attract wealth and abundance. Genuine tiger eye, look out, catches the light. Heavy, solid, the real deal. Black and gold beads all the way around. These keep selling out. Links down there, grab yours. Thank me later.</t>
         </is>
       </c>
-      <c r="R7" s="2" t="inlineStr">
+      <c r="S7" s="2" t="inlineStr">
         <is>
           <t>https://www.tiktok.com/@houseoframeau/video/7685441537894780190</t>
         </is>
       </c>
-      <c r="S7" s="2" t="inlineStr">
+      <c r="T7" s="2" t="inlineStr">
         <is>
           <t>https://shop.tiktok.com/us/pdp/arpurraina-money-attraction-necklace-tiger-eye-pendant/1732052135957598240</t>
         </is>
       </c>
-      <c r="T7" s="2" t="n">
+      <c r="U7" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="U7" s="2" t="n">
+      <c r="V7" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="V7" s="2" t="n">
+      <c r="W7" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="W7" s="2" t="inlineStr">
+      <c r="X7" s="2" t="inlineStr">
         <is>
           <t>houseoframeau account (not a Mymobileworld job folder)</t>
         </is>
       </c>
-      <c r="X7" s="2" t="inlineStr"/>
+      <c r="Y7" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Castor remix brief (4 x 15s, Grace's scripts + voice); all 5 Grace sellers are her own voice
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SJD4VaSy9o4r7BFp61EpGh
</commit_message>
<xml_diff>
--- a/grace/winners/winners.xlsx
+++ b/grace/winners/winners.xlsx
@@ -731,7 +731,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>likely Grace's own voice: posted words differ from our ElevenLabs file (to confirm)</t>
+          <t>Grace's own voice (Ralph 2026-10-20)</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>likely Grace's own voice: posted words differ from our ElevenLabs file (to confirm)</t>
+          <t>Grace's own voice (Ralph 2026-10-20)</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -953,7 +953,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>likely Grace's own voice: posted words differ from our ElevenLabs file (to confirm)</t>
+          <t>Grace's own voice (Ralph 2026-10-20)</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>likely Grace's own voice: posted words differ from our ElevenLabs file (to confirm)</t>
+          <t>Grace's own voice (Ralph 2026-10-20)</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sales tracker: BodyJ castor roll-on now 5 sales (Grace)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SJD4VaSy9o4r7BFp61EpGh
</commit_message>
<xml_diff>
--- a/grace/winners/winners.xlsx
+++ b/grace/winners/winners.xlsx
@@ -600,89 +600,89 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>2126</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>425</v>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Yes, by the brand (TikTok ad label)</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Grace's own voice (Ralph 2026-10-20)</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Hands + voiceover, AI, reply-to-comment video (marble bathroom, oil pour vs roll-on)</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>The only thing I hate about Castor oil is how thick and messy it is.</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Objection / Problem Callout</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>own line</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>Reply-to-comment sticker: "I think we all need castor oil" (@umi3728)</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>Castor oil is thick, messy and drips on your fingers, and the smell lingers.</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>A roll-on bottle with a rose quartz roller: no pouring, no oily fingers, put it exactly where you want (brows, cuticles, skin, hair).</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>Fastest start of the 6 (763 views a day). It replies to a real comment from her viral cradle-cap video, so it reaches people who already asked for castor oil (warm audience). Before/after messy pour vs clean roll is the proof. Grace's own wording ("freaking genius", "I'mma do y'all a favor") sounds like her, not an ad.</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>The only thing I hate about Castor oil is how thick and messy it is. And let's be for real, the smell isn't exactly something you want lingering all day. But if you know, you know, Castor oil is liquid gold. And this roll on. Freaking ingenious. No pouring, no oily fingers. Just roll it exactly where you want it. It's USDA organic, cold pressed and hexane free with a rose quartz roller. I'mma do y'all a favor and link it in the orange car. If you want condition brows, softer cuticles, moisturize skin and hair, growing longer, smoother, and shinier, you know what to do.</t>
+        </is>
+      </c>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@shewiththeglow/video/7697844264050511135</t>
+        </is>
+      </c>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>https://shop.tiktok.com/us/pdp/castor-castor-oil-roll-on-usda-organic-50ml-easy-application/1732039499743138513</t>
+        </is>
+      </c>
+      <c r="U2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="V2" s="2" t="n">
         <v>3</v>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>1578</v>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v>526</v>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Yes, by the brand (TikTok ad label)</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Grace's own voice (Ralph 2026-10-20)</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Hands + voiceover, AI, reply-to-comment video (marble bathroom, oil pour vs roll-on)</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>The only thing I hate about Castor oil is how thick and messy it is.</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>Objection / Problem Callout</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>own line</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>Reply-to-comment sticker: "I think we all need castor oil" (@umi3728)</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>Castor oil is thick, messy and drips on your fingers, and the smell lingers.</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>A roll-on bottle with a rose quartz roller: no pouring, no oily fingers, put it exactly where you want (brows, cuticles, skin, hair).</t>
-        </is>
-      </c>
-      <c r="Q2" s="2" t="inlineStr">
-        <is>
-          <t>Fastest start of the 6 (763 views a day). It replies to a real comment from her viral cradle-cap video, so it reaches people who already asked for castor oil (warm audience). Before/after messy pour vs clean roll is the proof. Grace's own wording ("freaking genius", "I'mma do y'all a favor") sounds like her, not an ad.</t>
-        </is>
-      </c>
-      <c r="R2" s="2" t="inlineStr">
-        <is>
-          <t>The only thing I hate about Castor oil is how thick and messy it is. And let's be for real, the smell isn't exactly something you want lingering all day. But if you know, you know, Castor oil is liquid gold. And this roll on. Freaking ingenious. No pouring, no oily fingers. Just roll it exactly where you want it. It's USDA organic, cold pressed and hexane free with a rose quartz roller. I'mma do y'all a favor and link it in the orange car. If you want condition brows, softer cuticles, moisturize skin and hair, growing longer, smoother, and shinier, you know what to do.</t>
-        </is>
-      </c>
-      <c r="S2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.tiktok.com/@shewiththeglow/video/7697844264050511135</t>
-        </is>
-      </c>
-      <c r="T2" s="2" t="inlineStr">
-        <is>
-          <t>https://shop.tiktok.com/us/pdp/castor-castor-oil-roll-on-usda-organic-50ml-easy-application/1732039499743138513</t>
-        </is>
-      </c>
-      <c r="U2" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="V2" s="2" t="n">
-        <v>2</v>
       </c>
       <c r="W2" s="2" t="n">
         <v>31</v>

</xml_diff>

<commit_message>
Sales tracker: add Vans sequin Authentic (1 sale, Grace)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SJD4VaSy9o4r7BFp61EpGh
</commit_message>
<xml_diff>
--- a/grace/winners/winners.xlsx
+++ b/grace/winners/winners.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y7"/>
+  <dimension ref="A1:Y8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -586,7 +586,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -596,17 +596,17 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>BodyJ4You Organic Oil Roll-On 1.7 oz - Castor, Rosehip, Jojoba, Argan, Coconut or Tea Tree - Rose Quartz Roller, Cold Pressed, Hexane Free</t>
+          <t>Vans Unisex Premium Authentic Low Top Shoe</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>2126</v>
+        <v>434</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>425</v>
+        <v>434</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -615,27 +615,27 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes (feet, legs and hands only)</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Grace's own voice (Ralph 2026-10-20)</t>
+          <t>Grace's voice, likely (her pattern; not confirmed for this one)</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Hands + voiceover, AI, reply-to-comment video (marble bathroom, oil pour vs roll-on)</t>
+          <t>Hands + feet + voiceover, AI: sequin close-up, shoes on, lacing up, held to camera at a crosswalk, white jeans, walking shots</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>The only thing I hate about Castor oil is how thick and messy it is.</t>
+          <t>Who told vans to come out with these sparkly low top?</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Objection / Problem Callout</t>
+          <t>Question (fun callout, own line)</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -645,51 +645,51 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Reply-to-comment sticker: "I think we all need castor oil" (@umi3728)</t>
+          <t>classic Vans with a plot twist 👀</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>Castor oil is thick, messy and drips on your fingers, and the smell lingers.</t>
+          <t>Classic Vans feel plain; wanting a sneaker with a little sparkle that still goes with everything.</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>A roll-on bottle with a rose quartz roller: no pouring, no oily fingers, put it exactly where you want (brows, cuticles, skin, hair).</t>
+          <t>Vans Premium Authentic with sequin checkerboard: the classic shape with shine, dressed up or casual, and comfortable.</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>Fastest start of the 6 (763 views a day). It replies to a real comment from her viral cradle-cap video, so it reaches people who already asked for castor oil (warm audience). Before/after messy pour vs clean roll is the proof. Grace's own wording ("freaking genius", "I'mma do y'all a favor") sounds like her, not an ad.</t>
+          <t>Known brand + a visual twist the eye catches in the first second (sequin close-up). The hook is a fun question with a compliment (whoever made that decision deserves a raise). Shows it worn many ways (white jeans, black pants, crosswalk, bag), so the viewer pictures her own outfit. Comfort answers the objection to fancy shoes. Watch: 'they're going to sell them out fast' is scarcity we can't back; leave it out of new versions.</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>The only thing I hate about Castor oil is how thick and messy it is. And let's be for real, the smell isn't exactly something you want lingering all day. But if you know, you know, Castor oil is liquid gold. And this roll on. Freaking ingenious. No pouring, no oily fingers. Just roll it exactly where you want it. It's USDA organic, cold pressed and hexane free with a rose quartz roller. I'mma do y'all a favor and link it in the orange car. If you want condition brows, softer cuticles, moisturize skin and hair, growing longer, smoother, and shinier, you know what to do.</t>
+          <t>Who told vans to come out with these sparkly low top? Because whoever made that decision deserves a raise. These are the premium authentic, and they really took the classic vans look and gave it a major upgrade. The sequence add just the right amount of shine without being over the top, so you can dress it up or keep it casual. And they're actually so comfortable, so you're getting the style and the comfort. These are new, but I wouldn't wait too long to grab them, because when the Shiny Girlies finds these, they're going to sell them out fast. Tap that orange car and get your size before they're gone.</t>
         </is>
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@shewiththeglow/video/7697844264050511135</t>
+          <t>https://www.tiktok.com/@shewiththeglow/video/7699252578239925535</t>
         </is>
       </c>
       <c r="T2" s="2" t="inlineStr">
         <is>
-          <t>https://shop.tiktok.com/us/pdp/castor-castor-oil-roll-on-usda-organic-50ml-easy-application/1732039499743138513</t>
+          <t>https://shop.tiktok.com/us/pdp/vans-unisex-premium-autc-low-top-shoe-lightweight-comfortable/1732459330963476520</t>
         </is>
       </c>
       <c r="U2" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="V2" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
-          <t>ugc/bodyj-castor-rollon/v2g (Grace's own script, word for word)</t>
+          <t>ugc/vans-sequin-authentic (10 AI videos, 2026-10-21)</t>
         </is>
       </c>
       <c r="Y2" s="2" t="inlineStr"/>
@@ -697,7 +697,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -707,17 +707,17 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>SoFyre Rodent Repellent Pouches (12 Pouches) – Natural Rodent Repellent with Peppermint &amp; Cinnamon Oils, Kids and Pets Safe Rodent Repellent, Long Lasting Rodent Control</t>
+          <t>BodyJ4You Organic Oil Roll-On 1.7 oz - Castor, Rosehip, Jojoba, Argan, Coconut or Tea Tree - Rose Quartz Roller, Cold Pressed, Hexane Free</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>2424</v>
+        <v>2126</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>2424</v>
+        <v>425</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -736,17 +736,17 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Hands + hand-free moving shots + voiceover, AI (pantry, garage, dog in hallway)</t>
+          <t>Hands + voiceover, AI, reply-to-comment video (marble bathroom, oil pour vs roll-on)</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Listen, when it gets cold outside, mice start looking for somewhere warm, and your house might be exactly what they're looking for.</t>
+          <t>The only thing I hate about Castor oil is how thick and messy it is.</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Time Pressure (Grace's rewording of H130)</t>
+          <t>Objection / Problem Callout</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -756,51 +756,51 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>the last thing you want in your pantry... 😳</t>
+          <t>Reply-to-comment sticker: "I think we all need castor oil" (@umi3728)</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>Mice moving in when it gets cold, and only finding out from droppings in the pantry; not wanting poison or traps around kids and pets.</t>
+          <t>Castor oil is thick, messy and drips on your fingers, and the smell lingers.</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>Peppermint + cinnamon oil pouches you drop where mice get in; no toxic chemicals, no traps to empty, 12 per bag, up to 3 months each.</t>
+          <t>A roll-on bottle with a rose quartz roller: no pouring, no oily fingers, put it exactly where you want (brows, cuticles, skin, hair).</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>Prevention before a deadline (cold weather) with a gross, visual payoff (droppings on the shelf). Removes the two big objections in one line each: safe around kids and pets, no traps to empty. The count + "grab two bags and do the whole house" pushes more than one unit.</t>
+          <t>Fastest start of the 6 (763 views a day). It replies to a real comment from her viral cradle-cap video, so it reaches people who already asked for castor oil (warm audience). Before/after messy pour vs clean roll is the proof. Grace's own wording ("freaking genius", "I'mma do y'all a favor") sounds like her, not an ad.</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>Listen, when it gets cold outside, mice start looking for somewhere warm, and your house might be exactly what they're looking for. And you won't even know until there are droppings in your pantry. So these let them out now. Just drop one wherever they get in. The pantry, under the sink, the garage, even the car. It's peppermint and cinnamon oil, so it smells fresh to us, but for mice, they don't like it. No toxic chemicals, so it's safe around kids and pets. And honestly, the best part, there's no traps to empty. There are 12 in the bag, and each one lasts up to three months. So grab two bags and do the whole house before the cold hits. I linked them below in the orange cart for you.</t>
+          <t>The only thing I hate about Castor oil is how thick and messy it is. And let's be for real, the smell isn't exactly something you want lingering all day. But if you know, you know, Castor oil is liquid gold. And this roll on. Freaking ingenious. No pouring, no oily fingers. Just roll it exactly where you want it. It's USDA organic, cold pressed and hexane free with a rose quartz roller. I'mma do y'all a favor and link it in the orange car. If you want condition brows, softer cuticles, moisturize skin and hair, growing longer, smoother, and shinier, you know what to do.</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@shewiththeglow/video/7696617399759555871</t>
+          <t>https://www.tiktok.com/@shewiththeglow/video/7697844264050511135</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>https://shop.tiktok.com/us/pdp/sofyre-mouse-repellent-pouches-natural-rodent-deterrent/1729505002971305054</t>
+          <t>https://shop.tiktok.com/us/pdp/castor-castor-oil-roll-on-usda-organic-50ml-easy-application/1732039499743138513</t>
         </is>
       </c>
       <c r="U3" s="2" t="n">
         <v>5</v>
       </c>
       <c r="V3" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="X3" s="2" t="inlineStr">
         <is>
-          <t>ugc/sofyre-rodent-pouches (r1 VO; Grace opened with "Listen," and reworded the hook when posting)</t>
+          <t>ugc/bodyj-castor-rollon/v2g (Grace's own script, word for word)</t>
         </is>
       </c>
       <c r="Y3" s="2" t="inlineStr"/>
@@ -818,21 +818,21 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Throw Hands Rock Paper Scissors Card Game - Fast-Paced, Chaotic Party Game for 2-8 Players, Ages 7+, 60-Second Family Game Night Game, Quick Travel Card Game for Kids, Teens &amp; Adults, Fun Group Game for Parties, Friends, Road Trips &amp; Vacations</t>
+          <t>SoFyre Rodent Repellent Pouches (12 Pouches) – Natural Rodent Repellent with Peppermint &amp; Cinnamon Oils, Kids and Pets Safe Rodent Repellent, Long Lasting Rodent Control</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>679</v>
+        <v>2424</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>679</v>
+        <v>2424</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes, by the brand (TikTok ad label)</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -847,17 +847,17 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Hands + voiceover, AI (overhead family table, cards being played)</t>
+          <t>Hands + hand-free moving shots + voiceover, AI (pantry, garage, dog in hallway)</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>You know game night is a wack when everyone's sitting around staring at their phones.</t>
+          <t>Listen, when it gets cold outside, mice start looking for somewhere warm, and your house might be exactly what they're looking for.</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Recognition (Grace's rewording of H062)</t>
+          <t>Time Pressure (Grace's rewording of H130)</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -867,51 +867,51 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>POV: you finally found a game everyone wants to play....</t>
+          <t>the last thing you want in your pantry... 😳</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>Game night dies: everyone on their phones, or the game drags so long people lose interest.</t>
+          <t>Mice moving in when it gets cold, and only finding out from droppings in the pantry; not wanting poison or traps around kids and pets.</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>A 60-second rock-paper-scissors card game, no waiting your turn, 2 to 8 players, easy to learn on the spot.</t>
+          <t>Peppermint + cinnamon oil pouches you drop where mice get in; no toxic chemicals, no traps to empty, 12 per bag, up to 3 months each.</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>Opens on a scene every family knows (phones at the table), then the rules are shown, not explained, so the viewer understands the game in 10 seconds. Thanksgiving gives the deadline, and "one for your house and one for your grandma's" sells two. Gift-able, low price.</t>
+          <t>Prevention before a deadline (cold weather) with a gross, visual payoff (droppings on the shelf). Removes the two big objections in one line each: safe around kids and pets, no traps to empty. The count + "grab two bags and do the whole house" pushes more than one unit.</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>You know game night is a wack when everyone's sitting around staring at their phones. Or when the game drags so long that everybody loses interest. This game fixes that real quick. It's called Throw Hands and think Rock, Paper, Scissors, but with cards and absolutely no waiting your turn. You slap down the card that beats the last one. Rock beat Scissors, paper beats rock, and Scissors beats paper. First person to get rid of all their cards wins. And with rounds lasting just 60 seconds, good luck just playing one round. Holiday fun is coming up, so grab one for your house and one for your grandma's. I linked it in the orange cart for you.</t>
+          <t>Listen, when it gets cold outside, mice start looking for somewhere warm, and your house might be exactly what they're looking for. And you won't even know until there are droppings in your pantry. So these let them out now. Just drop one wherever they get in. The pantry, under the sink, the garage, even the car. It's peppermint and cinnamon oil, so it smells fresh to us, but for mice, they don't like it. No toxic chemicals, so it's safe around kids and pets. And honestly, the best part, there's no traps to empty. There are 12 in the bag, and each one lasts up to three months. So grab two bags and do the whole house before the cold hits. I linked them below in the orange cart for you.</t>
         </is>
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@shewiththeglow/video/7696627904985304351</t>
+          <t>https://www.tiktok.com/@shewiththeglow/video/7696617399759555871</t>
         </is>
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>https://shop.tiktok.com/us/pdp/fast-fun-card-game-for-2-8-players-perfect-for-parties/1732271777612075081</t>
+          <t>https://shop.tiktok.com/us/pdp/sofyre-mouse-repellent-pouches-natural-rodent-deterrent/1729505002971305054</t>
         </is>
       </c>
       <c r="U4" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="V4" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>ugc/throw-hands-rps (r2b; Grace reworded the VO when posting)</t>
+          <t>ugc/sofyre-rodent-pouches (r1 VO; Grace opened with "Listen," and reworded the hook when posting)</t>
         </is>
       </c>
       <c r="Y4" s="2" t="inlineStr"/>
@@ -919,7 +919,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -929,21 +929,21 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Nasal Dilator – Starter Pack</t>
+          <t>Throw Hands Rock Paper Scissors Card Game - Fast-Paced, Chaotic Party Game for 2-8 Players, Ages 7+, 60-Second Family Game Night Game, Quick Travel Card Game for Kids, Teens &amp; Adults, Fun Group Game for Parties, Friends, Road Trips &amp; Vacations</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>3877</v>
+        <v>679</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>3877</v>
+        <v>679</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Yes, by the brand (TikTok ad label)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -958,71 +958,71 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Hands + voiceover, AI (bedroom at night, box + dilator close-ups)</t>
+          <t>Hands + voiceover, AI (overhead family table, cards being played)</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>This is for the people who always end up on the couch because somebody will not stop snoring.</t>
+          <t>You know game night is a wack when everyone's sitting around staring at their phones.</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>Recognition (Grace's rewording of H062)</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>H061</t>
+          <t>own line</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>POV: someone's snoring is ruining your sleep 😭</t>
+          <t>POV: you finally found a game everyone wants to play....</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>Losing sleep (or ending up on the couch) because the person next to you snores; nudging, earplugs and mouth tape did not fix it.</t>
+          <t>Game night dies: everyone on their phones, or the game drags so long people lose interest.</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>A tiny clear nasal dilator opens the nose so they snore less; the starter pack has all 3 sizes so you find the fit.</t>
+          <t>A 60-second rock-paper-scissors card game, no waiting your turn, 2 to 8 players, easy to learn on the spot.</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>Speaks to the person who suffers (the partner), not the snorer, so the buyer is the viewer. Lists what they already tried, then shows a small, cheap-feeling fix. Holiday shared rooms gives a reason to buy now. Most views of the 6 (3.9k) but the most views per sale: the broad pain gets reach, fewer of those viewers are ready to buy.</t>
+          <t>Opens on a scene every family knows (phones at the table), then the rules are shown, not explained, so the viewer understands the game in 10 seconds. Thanksgiving gives the deadline, and "one for your house and one for your grandma's" sells two. Gift-able, low price.</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>This is for the people who always end up on the couch because somebody will not stop snoring. You've tried nudging them, earplugs, and even mouth tape. This is mute, a tiny clear dilator that gently opens your nose. The starter pack has all three sizes and each one lasts up to 10 nights. Imagine actually getting some sleep instead of listening to snoring all night. And with the holiday travel coming up, this is worth packing for shared rooms. And you can find the mute starter pack a link below in the orange cart.</t>
+          <t>You know game night is a wack when everyone's sitting around staring at their phones. Or when the game drags so long that everybody loses interest. This game fixes that real quick. It's called Throw Hands and think Rock, Paper, Scissors, but with cards and absolutely no waiting your turn. You slap down the card that beats the last one. Rock beat Scissors, paper beats rock, and Scissors beats paper. First person to get rid of all their cards wins. And with rounds lasting just 60 seconds, good luck just playing one round. Holiday fun is coming up, so grab one for your house and one for your grandma's. I linked it in the orange cart for you.</t>
         </is>
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@shewiththeglow/video/7696231728855223582</t>
+          <t>https://www.tiktok.com/@shewiththeglow/video/7696627904985304351</t>
         </is>
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
-          <t>https://shop.tiktok.com/us/pdp/mute-nasal-dilator-starter-pack-reduces-snoring-3-sizes/1732240917356122930</t>
+          <t>https://shop.tiktok.com/us/pdp/fast-fun-card-game-for-2-8-players-perfect-for-parties/1732271777612075081</t>
         </is>
       </c>
       <c r="U5" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="V5" s="2" t="n">
         <v>1</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="X5" s="2" t="inlineStr">
         <is>
-          <t>ugc/mute-nasal-dilator (r4 VO; Grace dropped the 75% trial stat and the 2 a.m. joke when posting)</t>
+          <t>ugc/throw-hands-rps (r2b; Grace reworded the VO when posting)</t>
         </is>
       </c>
       <c r="Y5" s="2" t="inlineStr"/>
@@ -1040,17 +1040,17 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>【Buy there】Night Vision Driving Glasses Fit Over Glasses for Men Women Anti Glare Polarized HD Yellow Lens Unisex Design Enhance Night Drive Safety</t>
+          <t>Nasal Dilator – Starter Pack</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>463</v>
+        <v>3877</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>463</v>
+        <v>3877</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
@@ -1069,71 +1069,71 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Hands + voiceover, AI (POV through the windshield at night, glasses on the dash)</t>
+          <t>Hands + voiceover, AI (bedroom at night, box + dilator close-ups)</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>I wish someone thought of this sooner, because blinding headlights at night time, that's a whole different scary.</t>
+          <t>This is for the people who always end up on the couch because somebody will not stop snoring.</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Problem/Solution (close to H010)</t>
+          <t>Identity</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>own line</t>
+          <t>H061</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>blinding headlights at night are SCARY 😩</t>
+          <t>POV: someone's snoring is ruining your sleep 😭</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>Being blinded by bright headlights at night, squinting at the lane lines; worse if you already wear glasses.</t>
+          <t>Losing sleep (or ending up on the couch) because the person next to you snores; nudging, earplugs and mouth tape did not fix it.</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>Yellow-lens night driving glasses that fit over regular glasses, with side windows so glare cannot sneak in from the side.</t>
+          <t>A tiny clear nasal dilator opens the nose so they snore less; the starter pack has all 3 sizes so you find the fit.</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>Fewest views per sale of Grace's 5 (463 views, 1 sale). The fear is specific and visual (the white glare on screen), the viewer pictures their own drive home, and the clocks-go-back date (Nov 1) is real urgency. "Fit right over your regular ones" answers the glasses-wearer objection before they think it. Multi-unit ask: "grab one for a friend".</t>
+          <t>Speaks to the person who suffers (the partner), not the snorer, so the buyer is the viewer. Lists what they already tried, then shows a small, cheap-feeling fix. Holiday shared rooms gives a reason to buy now. Most views of the 6 (3.9k) but the most views per sale: the broad pain gets reach, fewer of those viewers are ready to buy.</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>I wish someone thought of this sooner, because blinding headlights at night time, that's a whole different scary. You're squinting at the lane lines, just hoping you're still in your lane. And wearing glasses that makes it even worse. These are night driving glasses that fit right over your regular ones. The yellow lenses are designed to help reduce glare from oncoming headlights. And there's a little window on each side so the glare can't even sneak in from the side. Now the clocks do go back on November 1st, which means darker drives home. Getting a pair of these is so worth it. And if you're feeling generous, grab one for a friend too. It's linked below in the orange cart.</t>
+          <t>This is for the people who always end up on the couch because somebody will not stop snoring. You've tried nudging them, earplugs, and even mouth tape. This is mute, a tiny clear dilator that gently opens your nose. The starter pack has all three sizes and each one lasts up to 10 nights. Imagine actually getting some sleep instead of listening to snoring all night. And with the holiday travel coming up, this is worth packing for shared rooms. And you can find the mute starter pack a link below in the orange cart.</t>
         </is>
       </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@shewiththeglow/video/7696285070046301470</t>
+          <t>https://www.tiktok.com/@shewiththeglow/video/7696231728855223582</t>
         </is>
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
-          <t>https://shop.tiktok.com/us/pdp/night-vision-driving-glasses-anti-glare-polarized-lenses/1731941490512139199</t>
+          <t>https://shop.tiktok.com/us/pdp/mute-nasal-dilator-starter-pack-reduces-snoring-3-sizes/1732240917356122930</t>
         </is>
       </c>
       <c r="U6" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="V6" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="X6" s="2" t="inlineStr">
         <is>
-          <t>ugc/night-driving-glasses/v2 (Grace's V1 script; she added "I wish someone thought of this sooner" at the start)</t>
+          <t>ugc/mute-nasal-dilator (r4 VO; Grace dropped the 75% trial stat and the 2 a.m. joke when posting)</t>
         </is>
       </c>
       <c r="Y6" s="2" t="inlineStr"/>
@@ -1141,56 +1141,56 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>@houseoframeau</t>
+          <t>@shewiththeglow</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>ARPURRAINA Tiger Eye Crystal Necklace - 69cm/27.1in Unisex Sweater Chain Healing Pendant, Crystal Jewellery, Men's Jewelry, Funky Unique Accessories, Attract Money Party-Theme Charm, Anniversary Gift</t>
+          <t>【Buy there】Night Vision Driving Glasses Fit Over Glasses for Men Women Anti Glare Polarized HD Yellow Lens Unisex Design Enhance Night Drive Safety</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>62</v>
+        <v>463</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>62</v>
+        <v>463</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes, by the brand (TikTok ad label)</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>No (AI man talking to camera)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>not known yet</t>
+          <t>Grace's own voice (Ralph 2026-10-20)</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Talking head, AI, lip-synced, home office, product worn and held to camera</t>
+          <t>Hands + voiceover, AI (POV through the windshield at night, glasses on the dash)</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>If this is your year to level up, do not scroll past this.</t>
+          <t>I wish someone thought of this sooner, because blinding headlights at night time, that's a whole different scary.</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Identity (callout)</t>
+          <t>Problem/Solution (close to H010)</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -1200,37 +1200,37 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>the necklace for your abundance era...✨</t>
+          <t>blinding headlights at night are SCARY 😩</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>Wanting to "level up" (money, confidence) this year and wanting something that reminds you every day.</t>
+          <t>Being blinded by bright headlights at night, squinting at the lane lines; worse if you already wear glasses.</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>A genuine tiger eye pendant on black and gold beads, an everyday reminder of abundance and confidence (identity product, not a fix).</t>
+          <t>Yellow-lens night driving glasses that fit over regular glasses, with side windows so glare cannot sneak in from the side.</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>1 sale on 61 views: tiny sample, so this is a lead, not proof. Short (13s) and fast. Identity hook ("if this is your year to level up") lets the buyer see themselves in it; close-ups show the stone catching the light (proof of quality), "heavy, solid, the real deal". Watch: "these keep selling out" is a scarcity claim we cannot back; keep it out of new versions unless the shop shows it.</t>
+          <t>Fewest views per sale of Grace's 5 (463 views, 1 sale). The fear is specific and visual (the white glare on screen), the viewer pictures their own drive home, and the clocks-go-back date (Nov 1) is real urgency. "Fit right over your regular ones" answers the glasses-wearer objection before they think it. Multi-unit ask: "grab one for a friend".</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>If this is your year to level up, do not scroll past this. This isn't just jewelry, it's your everyday reminder to attract wealth and abundance. Genuine tiger eye, look out, catches the light. Heavy, solid, the real deal. Black and gold beads all the way around. These keep selling out. Links down there, grab yours. Thank me later.</t>
+          <t>I wish someone thought of this sooner, because blinding headlights at night time, that's a whole different scary. You're squinting at the lane lines, just hoping you're still in your lane. And wearing glasses that makes it even worse. These are night driving glasses that fit right over your regular ones. The yellow lenses are designed to help reduce glare from oncoming headlights. And there's a little window on each side so the glare can't even sneak in from the side. Now the clocks do go back on November 1st, which means darker drives home. Getting a pair of these is so worth it. And if you're feeling generous, grab one for a friend too. It's linked below in the orange cart.</t>
         </is>
       </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@houseoframeau/video/7685441537894780190</t>
+          <t>https://www.tiktok.com/@shewiththeglow/video/7696285070046301470</t>
         </is>
       </c>
       <c r="T7" s="2" t="inlineStr">
         <is>
-          <t>https://shop.tiktok.com/us/pdp/arpurraina-money-attraction-necklace-tiger-eye-pendant/1732052135957598240</t>
+          <t>https://shop.tiktok.com/us/pdp/night-vision-driving-glasses-anti-glare-polarized-lenses/1731941490512139199</t>
         </is>
       </c>
       <c r="U7" s="2" t="n">
@@ -1240,14 +1240,125 @@
         <v>3</v>
       </c>
       <c r="W7" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="X7" s="2" t="inlineStr">
+        <is>
+          <t>ugc/night-driving-glasses/v2 (Grace's V1 script; she added "I wish someone thought of this sooner" at the start)</t>
+        </is>
+      </c>
+      <c r="Y7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>@houseoframeau</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>ARPURRAINA Tiger Eye Crystal Necklace - 69cm/27.1in Unisex Sweater Chain Healing Pendant, Crystal Jewellery, Men's Jewelry, Funky Unique Accessories, Attract Money Party-Theme Charm, Anniversary Gift</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>No (AI man talking to camera)</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>not known yet</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Talking head, AI, lip-synced, home office, product worn and held to camera</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>If this is your year to level up, do not scroll past this.</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Identity (callout)</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>own line</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>the necklace for your abundance era...✨</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>Wanting to "level up" (money, confidence) this year and wanting something that reminds you every day.</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>A genuine tiger eye pendant on black and gold beads, an everyday reminder of abundance and confidence (identity product, not a fix).</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t>1 sale on 61 views: tiny sample, so this is a lead, not proof. Short (13s) and fast. Identity hook ("if this is your year to level up") lets the buyer see themselves in it; close-ups show the stone catching the light (proof of quality), "heavy, solid, the real deal". Watch: "these keep selling out" is a scarcity claim we cannot back; keep it out of new versions unless the shop shows it.</t>
+        </is>
+      </c>
+      <c r="R8" s="2" t="inlineStr">
+        <is>
+          <t>If this is your year to level up, do not scroll past this. This isn't just jewelry, it's your everyday reminder to attract wealth and abundance. Genuine tiger eye, look out, catches the light. Heavy, solid, the real deal. Black and gold beads all the way around. These keep selling out. Links down there, grab yours. Thank me later.</t>
+        </is>
+      </c>
+      <c r="S8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@houseoframeau/video/7685441537894780190</t>
+        </is>
+      </c>
+      <c r="T8" s="2" t="inlineStr">
+        <is>
+          <t>https://shop.tiktok.com/us/pdp/arpurraina-money-attraction-necklace-tiger-eye-pendant/1732052135957598240</t>
+        </is>
+      </c>
+      <c r="U8" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="V8" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="W8" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="X7" s="2" t="inlineStr">
+      <c r="X8" s="2" t="inlineStr">
         <is>
           <t>houseoframeau account (not a Mymobileworld job folder)</t>
         </is>
       </c>
-      <c r="Y7" s="2" t="inlineStr"/>
+      <c r="Y8" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sales tracker: Vans voice = Grace's own; scarcity line left out (Ralph)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SJD4VaSy9o4r7BFp61EpGh
</commit_message>
<xml_diff>
--- a/grace/winners/winners.xlsx
+++ b/grace/winners/winners.xlsx
@@ -620,7 +620,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Grace's voice, likely (her pattern; not confirmed for this one)</t>
+          <t>Grace's own voice (Ralph 2026-10-24)</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -660,7 +660,7 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>Known brand + a visual twist the eye catches in the first second (sequin close-up). The hook is a fun question with a compliment (whoever made that decision deserves a raise). Shows it worn many ways (white jeans, black pants, crosswalk, bag), so the viewer pictures her own outfit. Comfort answers the objection to fancy shoes. Watch: 'they're going to sell them out fast' is scarcity we can't back; leave it out of new versions.</t>
+          <t>Known brand + a visual twist the eye catches in the first second (sequin close-up). The hook is a fun question with a compliment (whoever made that decision deserves a raise). Shows it worn many ways (white jeans, black pants, crosswalk, bag), so the viewer pictures her own outfit. Comfort answers the objection to fancy shoes. 'They're going to sell them out fast' is scarcity we can't back: left out of new versions (Ralph 2026-10-24).</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sales tracker: PRITECH face brush, 1 sale (Grace)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SJD4VaSy9o4r7BFp61EpGh
</commit_message>
<xml_diff>
--- a/grace/winners/winners.xlsx
+++ b/grace/winners/winners.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y8"/>
+  <dimension ref="A1:Y9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -586,7 +586,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -596,17 +596,17 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Vans Unisex Premium Authentic Low Top Shoe</t>
+          <t>Facial Cleansing Brush, PRITECH Heatable Vibrating Face Scrubber with Massage, Silicone Face Scrubber for Women &amp; Men, Electric Facial Cleanser for Deep Cleansing, Gentle Exfoliating (Pink)</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>434</v>
+        <v>1022</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>434</v>
+        <v>1022</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -615,27 +615,27 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Yes (feet, legs and hands only)</t>
+          <t>Yes (hands only)</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Grace's own voice (Ralph 2026-10-24)</t>
+          <t>Voiceover (Grace's own or ElevenLabs: not confirmed yet)</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Hands + feet + voiceover, AI: sequin close-up, shoes on, lacing up, held to camera at a crosswalk, white jeans, walking shots</t>
+          <t>Hands + voiceover, product demo: device lights up in hand on an acrylic stand, hands under the tap, makeup-stained towel, device on its charging base, lather on the cheek (no face), charging port close-up</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Who told vans to come out with these sparkly low top?</t>
+          <t>If you're not washing your face with a cleansing brush, what are you doing?</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Question (fun callout, own line)</t>
+          <t>Problem Callout (own line, no library match)</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -645,37 +645,37 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>classic Vans with a plot twist 👀</t>
+          <t>you're still washing you face.. without THIS???</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>Classic Vans feel plain; wanting a sneaker with a little sparkle that still goes with everything.</t>
+          <t>Washing with your hands leaves makeup and oil behind, and towels put bacteria back on your skin</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>Vans Premium Authentic with sequin checkerboard: the classic shape with shine, dressed up or casual, and comfortable.</t>
+          <t>Soft silicone bristles with 5 vibration settings clean deeper than hands, and the warming feature (up to 104 degrees) gives a spa feel at home</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>Known brand + a visual twist the eye catches in the first second (sequin close-up). The hook is a fun question with a compliment (whoever made that decision deserves a raise). Shows it worn many ways (white jeans, black pants, crosswalk, bag), so the viewer pictures her own outfit. Comfort answers the objection to fancy shoes. 'They're going to sell them out fast' is scarcity we can't back: left out of new versions (Ralph 2026-10-24).</t>
+          <t>Callout hook that makes the viewer feel behind (what are you doing?), plus the dirty towel as visible proof of the pain in the first 5 seconds. Three concrete features in one line, then a daily-habit justification (you do it every day, do it right). Short (20 s), product in hand from frame 0, Black Friday / gift hashtags in the season. Brand-promoted (ad label), so views are partly paid.</t>
         </is>
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>Who told vans to come out with these sparkly low top? Because whoever made that decision deserves a raise. These are the premium authentic, and they really took the classic vans look and gave it a major upgrade. The sequence add just the right amount of shine without being over the top, so you can dress it up or keep it casual. And they're actually so comfortable, so you're getting the style and the comfort. These are new, but I wouldn't wait too long to grab them, because when the Shiny Girlies finds these, they're going to sell them out fast. Tap that orange car and get your size before they're gone.</t>
+          <t>If you're not washing your face with a cleansing brush, what are you doing? Because using your hands leaves makeup and oil behind, and towels just transfer bacteria right back into your skin. This one has soft silicone bristles, five vibration settings, and a warming feature that heats up to 104 degrees, so you can get that little extra spa feel. And for something you do every single day, you might as well do it the right way. Go grab yours in an orange card before you forget about this.</t>
         </is>
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@shewiththeglow/video/7699252578239925535</t>
+          <t>https://www.tiktok.com/@shewiththeglow/video/7700400913759980831</t>
         </is>
       </c>
       <c r="T2" s="2" t="inlineStr">
         <is>
-          <t>https://shop.tiktok.com/us/pdp/vans-unisex-premium-autc-low-top-shoe-lightweight-comfortable/1732459330963476520</t>
+          <t>https://shop.tiktok.com/us/pdp/facial-cleansing-brush-pritech-heat-vibration-silicone-scrubber-for-deep-clean/1729468511278109083</t>
         </is>
       </c>
       <c r="U2" s="2" t="n">
@@ -685,11 +685,11 @@
         <v>0</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
-          <t>ugc/vans-sequin-authentic (10 AI videos, 2026-10-21)</t>
+          <t>Not made in our repo (no job folder): Grace's own production</t>
         </is>
       </c>
       <c r="Y2" s="2" t="inlineStr"/>
@@ -697,7 +697,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -707,17 +707,17 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>BodyJ4You Organic Oil Roll-On 1.7 oz - Castor, Rosehip, Jojoba, Argan, Coconut or Tea Tree - Rose Quartz Roller, Cold Pressed, Hexane Free</t>
+          <t>Vans Unisex Premium Authentic Low Top Shoe</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>2126</v>
+        <v>434</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>425</v>
+        <v>434</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -726,27 +726,27 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes (feet, legs and hands only)</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Grace's own voice (Ralph 2026-10-20)</t>
+          <t>Grace's own voice (Ralph 2026-10-24)</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Hands + voiceover, AI, reply-to-comment video (marble bathroom, oil pour vs roll-on)</t>
+          <t>Hands + feet + voiceover, AI: sequin close-up, shoes on, lacing up, held to camera at a crosswalk, white jeans, walking shots</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>The only thing I hate about Castor oil is how thick and messy it is.</t>
+          <t>Who told vans to come out with these sparkly low top?</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Objection / Problem Callout</t>
+          <t>Question (fun callout, own line)</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -756,51 +756,51 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Reply-to-comment sticker: "I think we all need castor oil" (@umi3728)</t>
+          <t>classic Vans with a plot twist 👀</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>Castor oil is thick, messy and drips on your fingers, and the smell lingers.</t>
+          <t>Classic Vans feel plain; wanting a sneaker with a little sparkle that still goes with everything.</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>A roll-on bottle with a rose quartz roller: no pouring, no oily fingers, put it exactly where you want (brows, cuticles, skin, hair).</t>
+          <t>Vans Premium Authentic with sequin checkerboard: the classic shape with shine, dressed up or casual, and comfortable.</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>Fastest start of the 6 (763 views a day). It replies to a real comment from her viral cradle-cap video, so it reaches people who already asked for castor oil (warm audience). Before/after messy pour vs clean roll is the proof. Grace's own wording ("freaking genius", "I'mma do y'all a favor") sounds like her, not an ad.</t>
+          <t>Known brand + a visual twist the eye catches in the first second (sequin close-up). The hook is a fun question with a compliment (whoever made that decision deserves a raise). Shows it worn many ways (white jeans, black pants, crosswalk, bag), so the viewer pictures her own outfit. Comfort answers the objection to fancy shoes. 'They're going to sell them out fast' is scarcity we can't back: left out of new versions (Ralph 2026-10-24).</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>The only thing I hate about Castor oil is how thick and messy it is. And let's be for real, the smell isn't exactly something you want lingering all day. But if you know, you know, Castor oil is liquid gold. And this roll on. Freaking ingenious. No pouring, no oily fingers. Just roll it exactly where you want it. It's USDA organic, cold pressed and hexane free with a rose quartz roller. I'mma do y'all a favor and link it in the orange car. If you want condition brows, softer cuticles, moisturize skin and hair, growing longer, smoother, and shinier, you know what to do.</t>
+          <t>Who told vans to come out with these sparkly low top? Because whoever made that decision deserves a raise. These are the premium authentic, and they really took the classic vans look and gave it a major upgrade. The sequence add just the right amount of shine without being over the top, so you can dress it up or keep it casual. And they're actually so comfortable, so you're getting the style and the comfort. These are new, but I wouldn't wait too long to grab them, because when the Shiny Girlies finds these, they're going to sell them out fast. Tap that orange car and get your size before they're gone.</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@shewiththeglow/video/7697844264050511135</t>
+          <t>https://www.tiktok.com/@shewiththeglow/video/7699252578239925535</t>
         </is>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>https://shop.tiktok.com/us/pdp/castor-castor-oil-roll-on-usda-organic-50ml-easy-application/1732039499743138513</t>
+          <t>https://shop.tiktok.com/us/pdp/vans-unisex-premium-autc-low-top-shoe-lightweight-comfortable/1732459330963476520</t>
         </is>
       </c>
       <c r="U3" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="V3" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="X3" s="2" t="inlineStr">
         <is>
-          <t>ugc/bodyj-castor-rollon/v2g (Grace's own script, word for word)</t>
+          <t>ugc/vans-sequin-authentic (10 AI videos, 2026-10-21)</t>
         </is>
       </c>
       <c r="Y3" s="2" t="inlineStr"/>
@@ -808,7 +808,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -818,17 +818,17 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>SoFyre Rodent Repellent Pouches (12 Pouches) – Natural Rodent Repellent with Peppermint &amp; Cinnamon Oils, Kids and Pets Safe Rodent Repellent, Long Lasting Rodent Control</t>
+          <t>BodyJ4You Organic Oil Roll-On 1.7 oz - Castor, Rosehip, Jojoba, Argan, Coconut or Tea Tree - Rose Quartz Roller, Cold Pressed, Hexane Free</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>2424</v>
+        <v>2126</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>2424</v>
+        <v>425</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
@@ -847,17 +847,17 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Hands + hand-free moving shots + voiceover, AI (pantry, garage, dog in hallway)</t>
+          <t>Hands + voiceover, AI, reply-to-comment video (marble bathroom, oil pour vs roll-on)</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Listen, when it gets cold outside, mice start looking for somewhere warm, and your house might be exactly what they're looking for.</t>
+          <t>The only thing I hate about Castor oil is how thick and messy it is.</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Time Pressure (Grace's rewording of H130)</t>
+          <t>Objection / Problem Callout</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -867,51 +867,51 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>the last thing you want in your pantry... 😳</t>
+          <t>Reply-to-comment sticker: "I think we all need castor oil" (@umi3728)</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>Mice moving in when it gets cold, and only finding out from droppings in the pantry; not wanting poison or traps around kids and pets.</t>
+          <t>Castor oil is thick, messy and drips on your fingers, and the smell lingers.</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>Peppermint + cinnamon oil pouches you drop where mice get in; no toxic chemicals, no traps to empty, 12 per bag, up to 3 months each.</t>
+          <t>A roll-on bottle with a rose quartz roller: no pouring, no oily fingers, put it exactly where you want (brows, cuticles, skin, hair).</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>Prevention before a deadline (cold weather) with a gross, visual payoff (droppings on the shelf). Removes the two big objections in one line each: safe around kids and pets, no traps to empty. The count + "grab two bags and do the whole house" pushes more than one unit.</t>
+          <t>Fastest start of the 6 (763 views a day). It replies to a real comment from her viral cradle-cap video, so it reaches people who already asked for castor oil (warm audience). Before/after messy pour vs clean roll is the proof. Grace's own wording ("freaking genius", "I'mma do y'all a favor") sounds like her, not an ad.</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>Listen, when it gets cold outside, mice start looking for somewhere warm, and your house might be exactly what they're looking for. And you won't even know until there are droppings in your pantry. So these let them out now. Just drop one wherever they get in. The pantry, under the sink, the garage, even the car. It's peppermint and cinnamon oil, so it smells fresh to us, but for mice, they don't like it. No toxic chemicals, so it's safe around kids and pets. And honestly, the best part, there's no traps to empty. There are 12 in the bag, and each one lasts up to three months. So grab two bags and do the whole house before the cold hits. I linked them below in the orange cart for you.</t>
+          <t>The only thing I hate about Castor oil is how thick and messy it is. And let's be for real, the smell isn't exactly something you want lingering all day. But if you know, you know, Castor oil is liquid gold. And this roll on. Freaking ingenious. No pouring, no oily fingers. Just roll it exactly where you want it. It's USDA organic, cold pressed and hexane free with a rose quartz roller. I'mma do y'all a favor and link it in the orange car. If you want condition brows, softer cuticles, moisturize skin and hair, growing longer, smoother, and shinier, you know what to do.</t>
         </is>
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@shewiththeglow/video/7696617399759555871</t>
+          <t>https://www.tiktok.com/@shewiththeglow/video/7697844264050511135</t>
         </is>
       </c>
       <c r="T4" s="2" t="inlineStr">
         <is>
-          <t>https://shop.tiktok.com/us/pdp/sofyre-mouse-repellent-pouches-natural-rodent-deterrent/1729505002971305054</t>
+          <t>https://shop.tiktok.com/us/pdp/castor-castor-oil-roll-on-usda-organic-50ml-easy-application/1732039499743138513</t>
         </is>
       </c>
       <c r="U4" s="2" t="n">
         <v>5</v>
       </c>
       <c r="V4" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>ugc/sofyre-rodent-pouches (r1 VO; Grace opened with "Listen," and reworded the hook when posting)</t>
+          <t>ugc/bodyj-castor-rollon/v2g (Grace's own script, word for word)</t>
         </is>
       </c>
       <c r="Y4" s="2" t="inlineStr"/>
@@ -929,21 +929,21 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Throw Hands Rock Paper Scissors Card Game - Fast-Paced, Chaotic Party Game for 2-8 Players, Ages 7+, 60-Second Family Game Night Game, Quick Travel Card Game for Kids, Teens &amp; Adults, Fun Group Game for Parties, Friends, Road Trips &amp; Vacations</t>
+          <t>SoFyre Rodent Repellent Pouches (12 Pouches) – Natural Rodent Repellent with Peppermint &amp; Cinnamon Oils, Kids and Pets Safe Rodent Repellent, Long Lasting Rodent Control</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>679</v>
+        <v>2424</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>679</v>
+        <v>2424</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes, by the brand (TikTok ad label)</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -958,17 +958,17 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Hands + voiceover, AI (overhead family table, cards being played)</t>
+          <t>Hands + hand-free moving shots + voiceover, AI (pantry, garage, dog in hallway)</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>You know game night is a wack when everyone's sitting around staring at their phones.</t>
+          <t>Listen, when it gets cold outside, mice start looking for somewhere warm, and your house might be exactly what they're looking for.</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Recognition (Grace's rewording of H062)</t>
+          <t>Time Pressure (Grace's rewording of H130)</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -978,51 +978,51 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>POV: you finally found a game everyone wants to play....</t>
+          <t>the last thing you want in your pantry... 😳</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>Game night dies: everyone on their phones, or the game drags so long people lose interest.</t>
+          <t>Mice moving in when it gets cold, and only finding out from droppings in the pantry; not wanting poison or traps around kids and pets.</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>A 60-second rock-paper-scissors card game, no waiting your turn, 2 to 8 players, easy to learn on the spot.</t>
+          <t>Peppermint + cinnamon oil pouches you drop where mice get in; no toxic chemicals, no traps to empty, 12 per bag, up to 3 months each.</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>Opens on a scene every family knows (phones at the table), then the rules are shown, not explained, so the viewer understands the game in 10 seconds. Thanksgiving gives the deadline, and "one for your house and one for your grandma's" sells two. Gift-able, low price.</t>
+          <t>Prevention before a deadline (cold weather) with a gross, visual payoff (droppings on the shelf). Removes the two big objections in one line each: safe around kids and pets, no traps to empty. The count + "grab two bags and do the whole house" pushes more than one unit.</t>
         </is>
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>You know game night is a wack when everyone's sitting around staring at their phones. Or when the game drags so long that everybody loses interest. This game fixes that real quick. It's called Throw Hands and think Rock, Paper, Scissors, but with cards and absolutely no waiting your turn. You slap down the card that beats the last one. Rock beat Scissors, paper beats rock, and Scissors beats paper. First person to get rid of all their cards wins. And with rounds lasting just 60 seconds, good luck just playing one round. Holiday fun is coming up, so grab one for your house and one for your grandma's. I linked it in the orange cart for you.</t>
+          <t>Listen, when it gets cold outside, mice start looking for somewhere warm, and your house might be exactly what they're looking for. And you won't even know until there are droppings in your pantry. So these let them out now. Just drop one wherever they get in. The pantry, under the sink, the garage, even the car. It's peppermint and cinnamon oil, so it smells fresh to us, but for mice, they don't like it. No toxic chemicals, so it's safe around kids and pets. And honestly, the best part, there's no traps to empty. There are 12 in the bag, and each one lasts up to three months. So grab two bags and do the whole house before the cold hits. I linked them below in the orange cart for you.</t>
         </is>
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@shewiththeglow/video/7696627904985304351</t>
+          <t>https://www.tiktok.com/@shewiththeglow/video/7696617399759555871</t>
         </is>
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
-          <t>https://shop.tiktok.com/us/pdp/fast-fun-card-game-for-2-8-players-perfect-for-parties/1732271777612075081</t>
+          <t>https://shop.tiktok.com/us/pdp/sofyre-mouse-repellent-pouches-natural-rodent-deterrent/1729505002971305054</t>
         </is>
       </c>
       <c r="U5" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="V5" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="X5" s="2" t="inlineStr">
         <is>
-          <t>ugc/throw-hands-rps (r2b; Grace reworded the VO when posting)</t>
+          <t>ugc/sofyre-rodent-pouches (r1 VO; Grace opened with "Listen," and reworded the hook when posting)</t>
         </is>
       </c>
       <c r="Y5" s="2" t="inlineStr"/>
@@ -1030,7 +1030,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -1040,21 +1040,21 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Nasal Dilator – Starter Pack</t>
+          <t>Throw Hands Rock Paper Scissors Card Game - Fast-Paced, Chaotic Party Game for 2-8 Players, Ages 7+, 60-Second Family Game Night Game, Quick Travel Card Game for Kids, Teens &amp; Adults, Fun Group Game for Parties, Friends, Road Trips &amp; Vacations</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>3877</v>
+        <v>679</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>3877</v>
+        <v>679</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Yes, by the brand (TikTok ad label)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -1069,71 +1069,71 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Hands + voiceover, AI (bedroom at night, box + dilator close-ups)</t>
+          <t>Hands + voiceover, AI (overhead family table, cards being played)</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>This is for the people who always end up on the couch because somebody will not stop snoring.</t>
+          <t>You know game night is a wack when everyone's sitting around staring at their phones.</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>Recognition (Grace's rewording of H062)</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>H061</t>
+          <t>own line</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>POV: someone's snoring is ruining your sleep 😭</t>
+          <t>POV: you finally found a game everyone wants to play....</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>Losing sleep (or ending up on the couch) because the person next to you snores; nudging, earplugs and mouth tape did not fix it.</t>
+          <t>Game night dies: everyone on their phones, or the game drags so long people lose interest.</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>A tiny clear nasal dilator opens the nose so they snore less; the starter pack has all 3 sizes so you find the fit.</t>
+          <t>A 60-second rock-paper-scissors card game, no waiting your turn, 2 to 8 players, easy to learn on the spot.</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>Speaks to the person who suffers (the partner), not the snorer, so the buyer is the viewer. Lists what they already tried, then shows a small, cheap-feeling fix. Holiday shared rooms gives a reason to buy now. Most views of the 6 (3.9k) but the most views per sale: the broad pain gets reach, fewer of those viewers are ready to buy.</t>
+          <t>Opens on a scene every family knows (phones at the table), then the rules are shown, not explained, so the viewer understands the game in 10 seconds. Thanksgiving gives the deadline, and "one for your house and one for your grandma's" sells two. Gift-able, low price.</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>This is for the people who always end up on the couch because somebody will not stop snoring. You've tried nudging them, earplugs, and even mouth tape. This is mute, a tiny clear dilator that gently opens your nose. The starter pack has all three sizes and each one lasts up to 10 nights. Imagine actually getting some sleep instead of listening to snoring all night. And with the holiday travel coming up, this is worth packing for shared rooms. And you can find the mute starter pack a link below in the orange cart.</t>
+          <t>You know game night is a wack when everyone's sitting around staring at their phones. Or when the game drags so long that everybody loses interest. This game fixes that real quick. It's called Throw Hands and think Rock, Paper, Scissors, but with cards and absolutely no waiting your turn. You slap down the card that beats the last one. Rock beat Scissors, paper beats rock, and Scissors beats paper. First person to get rid of all their cards wins. And with rounds lasting just 60 seconds, good luck just playing one round. Holiday fun is coming up, so grab one for your house and one for your grandma's. I linked it in the orange cart for you.</t>
         </is>
       </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@shewiththeglow/video/7696231728855223582</t>
+          <t>https://www.tiktok.com/@shewiththeglow/video/7696627904985304351</t>
         </is>
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
-          <t>https://shop.tiktok.com/us/pdp/mute-nasal-dilator-starter-pack-reduces-snoring-3-sizes/1732240917356122930</t>
+          <t>https://shop.tiktok.com/us/pdp/fast-fun-card-game-for-2-8-players-perfect-for-parties/1732271777612075081</t>
         </is>
       </c>
       <c r="U6" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="V6" s="2" t="n">
         <v>1</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="X6" s="2" t="inlineStr">
         <is>
-          <t>ugc/mute-nasal-dilator (r4 VO; Grace dropped the 75% trial stat and the 2 a.m. joke when posting)</t>
+          <t>ugc/throw-hands-rps (r2b; Grace reworded the VO when posting)</t>
         </is>
       </c>
       <c r="Y6" s="2" t="inlineStr"/>
@@ -1151,17 +1151,17 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>【Buy there】Night Vision Driving Glasses Fit Over Glasses for Men Women Anti Glare Polarized HD Yellow Lens Unisex Design Enhance Night Drive Safety</t>
+          <t>Nasal Dilator – Starter Pack</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>463</v>
+        <v>3877</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>463</v>
+        <v>3877</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
@@ -1180,71 +1180,71 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Hands + voiceover, AI (POV through the windshield at night, glasses on the dash)</t>
+          <t>Hands + voiceover, AI (bedroom at night, box + dilator close-ups)</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>I wish someone thought of this sooner, because blinding headlights at night time, that's a whole different scary.</t>
+          <t>This is for the people who always end up on the couch because somebody will not stop snoring.</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Problem/Solution (close to H010)</t>
+          <t>Identity</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>own line</t>
+          <t>H061</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>blinding headlights at night are SCARY 😩</t>
+          <t>POV: someone's snoring is ruining your sleep 😭</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>Being blinded by bright headlights at night, squinting at the lane lines; worse if you already wear glasses.</t>
+          <t>Losing sleep (or ending up on the couch) because the person next to you snores; nudging, earplugs and mouth tape did not fix it.</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>Yellow-lens night driving glasses that fit over regular glasses, with side windows so glare cannot sneak in from the side.</t>
+          <t>A tiny clear nasal dilator opens the nose so they snore less; the starter pack has all 3 sizes so you find the fit.</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>Fewest views per sale of Grace's 5 (463 views, 1 sale). The fear is specific and visual (the white glare on screen), the viewer pictures their own drive home, and the clocks-go-back date (Nov 1) is real urgency. "Fit right over your regular ones" answers the glasses-wearer objection before they think it. Multi-unit ask: "grab one for a friend".</t>
+          <t>Speaks to the person who suffers (the partner), not the snorer, so the buyer is the viewer. Lists what they already tried, then shows a small, cheap-feeling fix. Holiday shared rooms gives a reason to buy now. Most views of the 6 (3.9k) but the most views per sale: the broad pain gets reach, fewer of those viewers are ready to buy.</t>
         </is>
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>I wish someone thought of this sooner, because blinding headlights at night time, that's a whole different scary. You're squinting at the lane lines, just hoping you're still in your lane. And wearing glasses that makes it even worse. These are night driving glasses that fit right over your regular ones. The yellow lenses are designed to help reduce glare from oncoming headlights. And there's a little window on each side so the glare can't even sneak in from the side. Now the clocks do go back on November 1st, which means darker drives home. Getting a pair of these is so worth it. And if you're feeling generous, grab one for a friend too. It's linked below in the orange cart.</t>
+          <t>This is for the people who always end up on the couch because somebody will not stop snoring. You've tried nudging them, earplugs, and even mouth tape. This is mute, a tiny clear dilator that gently opens your nose. The starter pack has all three sizes and each one lasts up to 10 nights. Imagine actually getting some sleep instead of listening to snoring all night. And with the holiday travel coming up, this is worth packing for shared rooms. And you can find the mute starter pack a link below in the orange cart.</t>
         </is>
       </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@shewiththeglow/video/7696285070046301470</t>
+          <t>https://www.tiktok.com/@shewiththeglow/video/7696231728855223582</t>
         </is>
       </c>
       <c r="T7" s="2" t="inlineStr">
         <is>
-          <t>https://shop.tiktok.com/us/pdp/night-vision-driving-glasses-anti-glare-polarized-lenses/1731941490512139199</t>
+          <t>https://shop.tiktok.com/us/pdp/mute-nasal-dilator-starter-pack-reduces-snoring-3-sizes/1732240917356122930</t>
         </is>
       </c>
       <c r="U7" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="V7" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="X7" s="2" t="inlineStr">
         <is>
-          <t>ugc/night-driving-glasses/v2 (Grace's V1 script; she added "I wish someone thought of this sooner" at the start)</t>
+          <t>ugc/mute-nasal-dilator (r4 VO; Grace dropped the 75% trial stat and the 2 a.m. joke when posting)</t>
         </is>
       </c>
       <c r="Y7" s="2" t="inlineStr"/>
@@ -1252,56 +1252,56 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>@houseoframeau</t>
+          <t>@shewiththeglow</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>ARPURRAINA Tiger Eye Crystal Necklace - 69cm/27.1in Unisex Sweater Chain Healing Pendant, Crystal Jewellery, Men's Jewelry, Funky Unique Accessories, Attract Money Party-Theme Charm, Anniversary Gift</t>
+          <t>【Buy there】Night Vision Driving Glasses Fit Over Glasses for Men Women Anti Glare Polarized HD Yellow Lens Unisex Design Enhance Night Drive Safety</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>62</v>
+        <v>463</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>62</v>
+        <v>463</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes, by the brand (TikTok ad label)</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>No (AI man talking to camera)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>not known yet</t>
+          <t>Grace's own voice (Ralph 2026-10-20)</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Talking head, AI, lip-synced, home office, product worn and held to camera</t>
+          <t>Hands + voiceover, AI (POV through the windshield at night, glasses on the dash)</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>If this is your year to level up, do not scroll past this.</t>
+          <t>I wish someone thought of this sooner, because blinding headlights at night time, that's a whole different scary.</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Identity (callout)</t>
+          <t>Problem/Solution (close to H010)</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -1311,37 +1311,37 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>the necklace for your abundance era...✨</t>
+          <t>blinding headlights at night are SCARY 😩</t>
         </is>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>Wanting to "level up" (money, confidence) this year and wanting something that reminds you every day.</t>
+          <t>Being blinded by bright headlights at night, squinting at the lane lines; worse if you already wear glasses.</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>A genuine tiger eye pendant on black and gold beads, an everyday reminder of abundance and confidence (identity product, not a fix).</t>
+          <t>Yellow-lens night driving glasses that fit over regular glasses, with side windows so glare cannot sneak in from the side.</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>1 sale on 61 views: tiny sample, so this is a lead, not proof. Short (13s) and fast. Identity hook ("if this is your year to level up") lets the buyer see themselves in it; close-ups show the stone catching the light (proof of quality), "heavy, solid, the real deal". Watch: "these keep selling out" is a scarcity claim we cannot back; keep it out of new versions unless the shop shows it.</t>
+          <t>Fewest views per sale of Grace's 5 (463 views, 1 sale). The fear is specific and visual (the white glare on screen), the viewer pictures their own drive home, and the clocks-go-back date (Nov 1) is real urgency. "Fit right over your regular ones" answers the glasses-wearer objection before they think it. Multi-unit ask: "grab one for a friend".</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>If this is your year to level up, do not scroll past this. This isn't just jewelry, it's your everyday reminder to attract wealth and abundance. Genuine tiger eye, look out, catches the light. Heavy, solid, the real deal. Black and gold beads all the way around. These keep selling out. Links down there, grab yours. Thank me later.</t>
+          <t>I wish someone thought of this sooner, because blinding headlights at night time, that's a whole different scary. You're squinting at the lane lines, just hoping you're still in your lane. And wearing glasses that makes it even worse. These are night driving glasses that fit right over your regular ones. The yellow lenses are designed to help reduce glare from oncoming headlights. And there's a little window on each side so the glare can't even sneak in from the side. Now the clocks do go back on November 1st, which means darker drives home. Getting a pair of these is so worth it. And if you're feeling generous, grab one for a friend too. It's linked below in the orange cart.</t>
         </is>
       </c>
       <c r="S8" s="2" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@houseoframeau/video/7685441537894780190</t>
+          <t>https://www.tiktok.com/@shewiththeglow/video/7696285070046301470</t>
         </is>
       </c>
       <c r="T8" s="2" t="inlineStr">
         <is>
-          <t>https://shop.tiktok.com/us/pdp/arpurraina-money-attraction-necklace-tiger-eye-pendant/1732052135957598240</t>
+          <t>https://shop.tiktok.com/us/pdp/night-vision-driving-glasses-anti-glare-polarized-lenses/1731941490512139199</t>
         </is>
       </c>
       <c r="U8" s="2" t="n">
@@ -1351,14 +1351,125 @@
         <v>3</v>
       </c>
       <c r="W8" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="X8" s="2" t="inlineStr">
+        <is>
+          <t>ugc/night-driving-glasses/v2 (Grace's V1 script; she added "I wish someone thought of this sooner" at the start)</t>
+        </is>
+      </c>
+      <c r="Y8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>@houseoframeau</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>ARPURRAINA Tiger Eye Crystal Necklace - 69cm/27.1in Unisex Sweater Chain Healing Pendant, Crystal Jewellery, Men's Jewelry, Funky Unique Accessories, Attract Money Party-Theme Charm, Anniversary Gift</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>No (AI man talking to camera)</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>not known yet</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Talking head, AI, lip-synced, home office, product worn and held to camera</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>If this is your year to level up, do not scroll past this.</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Identity (callout)</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>own line</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>the necklace for your abundance era...✨</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>Wanting to "level up" (money, confidence) this year and wanting something that reminds you every day.</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>A genuine tiger eye pendant on black and gold beads, an everyday reminder of abundance and confidence (identity product, not a fix).</t>
+        </is>
+      </c>
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>1 sale on 61 views: tiny sample, so this is a lead, not proof. Short (13s) and fast. Identity hook ("if this is your year to level up") lets the buyer see themselves in it; close-ups show the stone catching the light (proof of quality), "heavy, solid, the real deal". Watch: "these keep selling out" is a scarcity claim we cannot back; keep it out of new versions unless the shop shows it.</t>
+        </is>
+      </c>
+      <c r="R9" s="2" t="inlineStr">
+        <is>
+          <t>If this is your year to level up, do not scroll past this. This isn't just jewelry, it's your everyday reminder to attract wealth and abundance. Genuine tiger eye, look out, catches the light. Heavy, solid, the real deal. Black and gold beads all the way around. These keep selling out. Links down there, grab yours. Thank me later.</t>
+        </is>
+      </c>
+      <c r="S9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@houseoframeau/video/7685441537894780190</t>
+        </is>
+      </c>
+      <c r="T9" s="2" t="inlineStr">
+        <is>
+          <t>https://shop.tiktok.com/us/pdp/arpurraina-money-attraction-necklace-tiger-eye-pendant/1732052135957598240</t>
+        </is>
+      </c>
+      <c r="U9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="V9" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="W9" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="X8" s="2" t="inlineStr">
+      <c r="X9" s="2" t="inlineStr">
         <is>
           <t>houseoframeau account (not a Mymobileworld job folder)</t>
         </is>
       </c>
-      <c r="Y8" s="2" t="inlineStr"/>
+      <c r="Y9" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sales tracker: PRITECH sale = Grace's re-edit of our V1 + her Oct 23 video, her voice (Ralph)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SJD4VaSy9o4r7BFp61EpGh
</commit_message>
<xml_diff>
--- a/grace/winners/winners.xlsx
+++ b/grace/winners/winners.xlsx
@@ -620,12 +620,12 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Voiceover (Grace's own or ElevenLabs: not confirmed yet)</t>
+          <t>Grace's own voice, reused from her Oct 23 video https://www.tiktok.com/t/ZPLAonsjU/ (Ralph 2026-10-28)</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Hands + voiceover, product demo: device lights up in hand on an acrylic stand, hands under the tap, makeup-stained towel, device on its charging base, lather on the cheek (no face), charging port close-up</t>
+          <t>Grace's re-edit: clips from her Oct 23 PRITECH video plus our AI V1 footage (hands only): brush lights up in hand on an acrylic stand, hands under the tap, makeup-stained towel, brush on its charging base, lather on the cheek (no face), charging port close-up</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -689,10 +689,14 @@
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
-          <t>Not made in our repo (no job folder): Grace's own production</t>
-        </is>
-      </c>
-      <c r="Y2" s="2" t="inlineStr"/>
+          <t>ugc/pritech-cleansing-brush (our V1, 2026-10-24); Grace mixed its clips with her Oct 23 video (Ralph 2026-10-28)</t>
+        </is>
+      </c>
+      <c r="Y2" s="2" t="inlineStr">
+        <is>
+          <t>Same script and voice as her Oct 23 video (1,327 views, no sale reported); new footage mix + new caption got the sale</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">

</xml_diff>